<commit_message>
Deployed de4d91f with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -818,10 +818,10 @@
         <v>23</v>
       </c>
       <c r="M7" t="n">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="N7" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1154,7 +1154,7 @@
         <v>4</v>
       </c>
       <c r="M13" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="N13" t="n">
         <v>4</v>
@@ -1210,10 +1210,10 @@
         <v>57</v>
       </c>
       <c r="M14" t="n">
-        <v>140</v>
+        <v>114</v>
       </c>
       <c r="N14" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
@@ -1266,10 +1266,10 @@
         <v>26</v>
       </c>
       <c r="M15" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="N15" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sharma_2018_BisphenolA_Human</t>
+          <t>Sharma2018_BPA_Human</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Moreau_BPA_Human</t>
+          <t>Moreau2025_BPA_Human</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Deepika_2022_BisphenolA_Human</t>
+          <t>Deepika2022_BPA_Human</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2442,10 +2442,10 @@
         <v>37</v>
       </c>
       <c r="M36" t="n">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="N36" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Loizou2022_BisphenolA_Human</t>
+          <t>Loizou2022_BPA_Human</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2834,10 +2834,10 @@
         <v>7</v>
       </c>
       <c r="M43" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N43" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44">
@@ -3058,10 +3058,10 @@
         <v>7</v>
       </c>
       <c r="M47" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N47" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48">
@@ -3114,10 +3114,10 @@
         <v>7</v>
       </c>
       <c r="M48" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N48" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
Deployed 2e04e83 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,60 +429,65 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>route</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>chemical_group</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>report_path</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>compartments</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>num_compartments</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>num_compartments_unannotated</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>num_species</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>num_species_unannotated</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>num_parameters</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>num_parameters_unannotated</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>num_unit_consistency_errors</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>num_unit_consistency_warnings</t>
         </is>
@@ -491,673 +496,733 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Notenboom.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Notenboom2023_DON_Human</t>
+          <t>Chen2022_PFOS_Human</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Lumen;Liver;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>4</v>
+          <t>./models/oral/PFAS/Chen/summary.md</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+        </is>
       </c>
       <c r="H2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>6</v>
       </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
       <c r="K2" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="M2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="O2" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mendez_Catala.sbml</t>
+          <t>ChouLin.sbml</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mandez_Catal_2021_Human_PBK</t>
+          <t>Chou_Lin2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>ChouLin</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>14</v>
+          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+        </is>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="K3" t="n">
-        <v>87</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
         <v>29</v>
       </c>
       <c r="M3" t="n">
-        <v>59</v>
+        <v>7</v>
       </c>
       <c r="N3" t="n">
-        <v>32</v>
+        <v>10</v>
+      </c>
+      <c r="O3" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wang.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Wang2023_DON_Human</t>
+          <t>Deepika2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>8</v>
+          <t>./models/oral/PFAS/Deepika/summary.md</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest</t>
+        </is>
       </c>
       <c r="H4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>25</v>
+      </c>
+      <c r="M4" t="n">
         <v>1</v>
       </c>
-      <c r="I4" t="n">
-        <v>9</v>
-      </c>
-      <c r="J4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K4" t="n">
-        <v>48</v>
-      </c>
-      <c r="L4" t="n">
-        <v>17</v>
-      </c>
-      <c r="M4" t="n">
-        <v>7</v>
-      </c>
       <c r="N4" t="n">
-        <v>17</v>
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval.sbml</t>
+          <t>LoccisanoPFOA.sbml</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>GilbertSandoval</t>
+          <t>Loccisano2011_PFOA_Human</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>LoccisanoPFOA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>13</v>
+          <t>./models/oral/PFAS/Loccisano_PFOA/summary.md</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest</t>
+        </is>
       </c>
       <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>25</v>
+      </c>
+      <c r="M5" t="n">
         <v>1</v>
       </c>
-      <c r="I5" t="n">
-        <v>15</v>
-      </c>
-      <c r="J5" t="n">
-        <v>11</v>
-      </c>
-      <c r="K5" t="n">
-        <v>46</v>
-      </c>
-      <c r="L5" t="n">
-        <v>18</v>
-      </c>
-      <c r="M5" t="n">
-        <v>40</v>
-      </c>
       <c r="N5" t="n">
-        <v>9</v>
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mukherjee.sbml</t>
+          <t>Worley.sbml</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mukherjee2014_Human_PBK</t>
+          <t>Worley2017_PFOA_Human</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Worley</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>12</v>
+          <t>./models/oral/PFAS/Worley/summary.md</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+        </is>
       </c>
       <c r="H6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" t="n">
         <v>2</v>
       </c>
-      <c r="I6" t="n">
-        <v>16</v>
-      </c>
-      <c r="J6" t="n">
-        <v>11</v>
-      </c>
-      <c r="K6" t="n">
-        <v>51</v>
-      </c>
       <c r="L6" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="M6" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="N6" t="n">
-        <v>33</v>
+        <v>10</v>
+      </c>
+      <c r="O6" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Timchalk.sbml</t>
+          <t>LoccisanoPFOS.sbml</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Timchalk2002_Chlorpyrifos_Human</t>
+          <t>Loccisano2011_PFOS_Human</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>LoccisanoPFOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
+          <t>./models/oral/PFAS/Loccisano_PFOS/summary.md</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>25</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
         <v>3</v>
-      </c>
-      <c r="H7" t="n">
-        <v>3</v>
-      </c>
-      <c r="I7" t="n">
-        <v>5</v>
-      </c>
-      <c r="J7" t="n">
-        <v>5</v>
-      </c>
-      <c r="K7" t="n">
-        <v>23</v>
-      </c>
-      <c r="L7" t="n">
-        <v>23</v>
-      </c>
-      <c r="M7" t="n">
-        <v>46</v>
-      </c>
-      <c r="N7" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mallick.sbml</t>
+          <t>Husoy.sbml</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mallick2020_Pyrethroids_Human</t>
+          <t>Husoy2024_PFOA_Human</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Husoy</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Mallick/summary.md</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>6</v>
+          <t>./models/oral/PFAS/Husoy/summary.md</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest;Feces</t>
+        </is>
       </c>
       <c r="H8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="M8" t="n">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="N8" t="n">
-        <v>35</v>
+        <v>2</v>
+      </c>
+      <c r="O8" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Tonnelier.sbml</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chen_Fenitrothion_Human</t>
+          <t>Tonnelier2012_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Tonnelier</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>./models/oral/Pesticides/Chen/summary.md</t>
-        </is>
-      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>5</v>
+          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
+        </is>
       </c>
       <c r="H9" t="n">
         <v>5</v>
       </c>
       <c r="I9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K9" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="L9" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="M9" t="n">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="N9" t="n">
-        <v>24</v>
+        <v>58</v>
+      </c>
+      <c r="O9" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>Chen_Fenitrothion_Human</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
+          <t>./models/oral/Pesticides/Chen/summary.md</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" t="n">
         <v>7</v>
       </c>
-      <c r="H10" t="n">
+      <c r="K10" t="n">
         <v>7</v>
       </c>
-      <c r="I10" t="n">
-        <v>9</v>
-      </c>
-      <c r="J10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K10" t="n">
-        <v>37</v>
-      </c>
       <c r="L10" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="M10" t="n">
-        <v>108</v>
+        <v>31</v>
       </c>
       <c r="N10" t="n">
-        <v>33</v>
+        <v>88</v>
+      </c>
+      <c r="O10" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl.sbml</t>
+          <t>Zhao.sbml</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>Zhao2019_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Zhao</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
-        </is>
-      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
+          <t>./models/oral/Pesticides/Zhao/summary.md</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Gut;Liver;Blood;Rest</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" t="n">
         <v>7</v>
       </c>
-      <c r="H11" t="n">
+      <c r="K11" t="n">
         <v>7</v>
       </c>
-      <c r="I11" t="n">
-        <v>9</v>
-      </c>
-      <c r="J11" t="n">
-        <v>9</v>
-      </c>
-      <c r="K11" t="n">
-        <v>37</v>
-      </c>
       <c r="L11" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="M11" t="n">
-        <v>108</v>
+        <v>26</v>
       </c>
       <c r="N11" t="n">
-        <v>33</v>
+        <v>52</v>
+      </c>
+      <c r="O11" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tonnelier.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Tonnelier2012_Chlorpyrifos_Human</t>
+          <t>Bouchard2010_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
-        </is>
-      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>5</v>
+          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Gut;Blood;Rest</t>
+        </is>
       </c>
       <c r="H12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="M12" t="n">
-        <v>58</v>
+        <v>4</v>
       </c>
       <c r="N12" t="n">
-        <v>18</v>
+        <v>8</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bouchard.sbml</t>
+          <t>Godin.sbml</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bouchard2010_Chlorpyrifos_Human</t>
+          <t>Godin_Pyrethroid_Human</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Godin</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
-        </is>
-      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Gut;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>3</v>
+          <t>./models/oral/Pesticides/Godin/summary.md</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
+        </is>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I13" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L13" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="M13" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>106</v>
+      </c>
+      <c r="O13" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="14">
@@ -1173,2119 +1238,2309 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Zwartsen</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
         </is>
-      </c>
-      <c r="G14" t="n">
-        <v>5</v>
       </c>
       <c r="H14" t="n">
         <v>5</v>
       </c>
       <c r="I14" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J14" t="n">
         <v>7</v>
       </c>
       <c r="K14" t="n">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="L14" t="n">
         <v>57</v>
       </c>
       <c r="M14" t="n">
+        <v>57</v>
+      </c>
+      <c r="N14" t="n">
         <v>114</v>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Zhao.sbml</t>
+          <t>Moreau_Carbaryl.sbml</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Zhao2019_Chlorpyrifos_Human</t>
+          <t>Moreau_Deltamethrin_Human</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Moreau_Deltamethrin</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>./models/oral/Pesticides/Zhao/summary.md</t>
-        </is>
-      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>4</v>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+        </is>
       </c>
       <c r="H15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I15" t="n">
         <v>7</v>
       </c>
       <c r="J15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K15" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="L15" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="M15" t="n">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="N15" t="n">
-        <v>17</v>
+        <v>108</v>
+      </c>
+      <c r="O15" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Wei.sbml</t>
+          <t>Moreau_Deltamethrin.sbml</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Wei_Permethrin_Human</t>
+          <t>Moreau_Deltamethrin_Human</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Moreau_Deltamethrin</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>./models/oral/Pesticides/Wei/summary.md</t>
-        </is>
-      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I16" t="n">
+        <v>7</v>
+      </c>
+      <c r="J16" t="n">
         <v>9</v>
       </c>
-      <c r="H16" t="n">
+      <c r="K16" t="n">
         <v>9</v>
       </c>
-      <c r="I16" t="n">
-        <v>11</v>
-      </c>
-      <c r="J16" t="n">
-        <v>11</v>
-      </c>
-      <c r="K16" t="n">
-        <v>31</v>
-      </c>
       <c r="L16" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="M16" t="n">
-        <v>104</v>
+        <v>37</v>
       </c>
       <c r="N16" t="n">
-        <v>32</v>
+        <v>108</v>
+      </c>
+      <c r="O16" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Godin.sbml</t>
+          <t>Timchalk.sbml</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Godin_Pyrethroid_Human</t>
+          <t>Timchalk2002_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Timchalk</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>Pesticides</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>./models/oral/Pesticides/Godin/summary.md</t>
-        </is>
-      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>8</v>
+          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Liver;Blood;Rest</t>
+        </is>
       </c>
       <c r="H17" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I17" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J17" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K17" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="L17" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="M17" t="n">
-        <v>106</v>
+        <v>23</v>
       </c>
       <c r="N17" t="n">
-        <v>36</v>
+        <v>46</v>
+      </c>
+      <c r="O17" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb_Human_Male</t>
+          <t>Wei_Permethrin_Human</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty_2000_Pb/summary.md</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>3</v>
+          <t>./models/oral/Pesticides/Wei/summary.md</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
+        </is>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I18" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K18" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="M18" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="N18" t="n">
-        <v>6</v>
+        <v>104</v>
+      </c>
+      <c r="O18" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BechauxCd_Female.sbml</t>
+          <t>Mallick.sbml</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Male</t>
+          <t>Mallick2020_Pyrethroids_Human</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Mallick</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux_Cd/summary.md</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>9</v>
+          <t>./models/oral/Pesticides/Mallick/summary.md</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
+        </is>
       </c>
       <c r="H19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I19" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K19" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L19" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="M19" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="N19" t="n">
-        <v>10</v>
+        <v>100</v>
+      </c>
+      <c r="O19" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BechauxCd_Male.sbml</t>
+          <t>Teeguarden.sbml</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Male</t>
+          <t>Teeguarden2005_BPA_Human</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Teeguarden</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux_Cd/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
+          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>GILumen;Liver;Blood;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>8</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>30</v>
+      </c>
+      <c r="M20" t="n">
+        <v>6</v>
+      </c>
+      <c r="N20" t="n">
+        <v>12</v>
+      </c>
+      <c r="O20" t="n">
         <v>9</v>
-      </c>
-      <c r="H20" t="n">
-        <v>3</v>
-      </c>
-      <c r="I20" t="n">
-        <v>9</v>
-      </c>
-      <c r="J20" t="n">
-        <v>3</v>
-      </c>
-      <c r="K20" t="n">
-        <v>15</v>
-      </c>
-      <c r="L20" t="n">
-        <v>12</v>
-      </c>
-      <c r="M20" t="n">
-        <v>9</v>
-      </c>
-      <c r="N20" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ElMasri_2008_As.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ElMasri2008_As_Human_Male</t>
+          <t>Deepika2022_BPA_Human</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/ElMasri_As/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
+          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" t="n">
+        <v>2</v>
+      </c>
+      <c r="J21" t="n">
         <v>8</v>
       </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>32</v>
-      </c>
-      <c r="J21" t="n">
-        <v>2</v>
-      </c>
       <c r="K21" t="n">
-        <v>78</v>
+        <v>4</v>
       </c>
       <c r="L21" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="M21" t="n">
-        <v>107</v>
+        <v>37</v>
       </c>
       <c r="N21" t="n">
-        <v>19</v>
+        <v>76</v>
+      </c>
+      <c r="O21" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RuizCd_Male.sbml</t>
+          <t>Sharma.sbml</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>Sharma2018_BPA_Human</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz_Cd/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
+          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>5</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>8</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>38</v>
+      </c>
+      <c r="M22" t="n">
+        <v>5</v>
+      </c>
+      <c r="N22" t="n">
+        <v>17</v>
+      </c>
+      <c r="O22" t="n">
         <v>9</v>
-      </c>
-      <c r="H22" t="n">
-        <v>7</v>
-      </c>
-      <c r="I22" t="n">
-        <v>9</v>
-      </c>
-      <c r="J22" t="n">
-        <v>5</v>
-      </c>
-      <c r="K22" t="n">
-        <v>15</v>
-      </c>
-      <c r="L22" t="n">
-        <v>14</v>
-      </c>
-      <c r="M22" t="n">
-        <v>68</v>
-      </c>
-      <c r="N22" t="n">
-        <v>22</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RuizCd_Female.sbml</t>
+          <t>Shin.sbml</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>Shin2004_BPA_Human</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Shin</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz_Cd/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>9</v>
+          <t>./models/oral/Bisphenols/Shin/summary.md</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
+        </is>
       </c>
       <c r="H23" t="n">
         <v>7</v>
       </c>
       <c r="I23" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K23" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="L23" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="M23" t="n">
-        <v>68</v>
+        <v>7</v>
       </c>
       <c r="N23" t="n">
-        <v>22</v>
+        <v>2</v>
+      </c>
+      <c r="O23" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ou2018_Hg.sbml</t>
+          <t>Yang.sbml</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ou2018_Hg_Human</t>
+          <t>Yang2015_BPA_Human</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Yang</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ou_2018/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
+          <t>./models/oral/Bisphenols/Yang/summary.md</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
         <v>7</v>
       </c>
-      <c r="H24" t="n">
+      <c r="I24" t="n">
         <v>0</v>
       </c>
-      <c r="I24" t="n">
-        <v>9</v>
-      </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="K24" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="M24" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="N24" t="n">
-        <v>4</v>
+        <v>71</v>
+      </c>
+      <c r="O24" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Clewell1999_Hg.sbml</t>
+          <t>Moreau.sbml</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Clewell_Hg_Human</t>
+          <t>Moreau2025_BPA_Human</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Moreau</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Clewell_Hg/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
+          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
         <v>7</v>
       </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
       <c r="I25" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" t="n">
         <v>9</v>
       </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
       <c r="K25" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="M25" t="n">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="N25" t="n">
-        <v>2</v>
+        <v>75</v>
+      </c>
+      <c r="O25" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PouillotCd.sbml</t>
+          <t>Mielke.sbml</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Male</t>
+          <t>Mielke2009_BPA_Human</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Mielke</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Pouillot_Cd/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
+          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Gut;Liver;Blood;Rest</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>4</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>6</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>22</v>
+      </c>
+      <c r="M26" t="n">
+        <v>2</v>
+      </c>
+      <c r="N26" t="n">
         <v>9</v>
       </c>
-      <c r="H26" t="n">
-        <v>2</v>
-      </c>
-      <c r="I26" t="n">
-        <v>9</v>
-      </c>
-      <c r="J26" t="n">
-        <v>2</v>
-      </c>
-      <c r="K26" t="n">
-        <v>14</v>
-      </c>
-      <c r="L26" t="n">
-        <v>12</v>
-      </c>
-      <c r="M26" t="n">
-        <v>7</v>
-      </c>
-      <c r="N26" t="n">
-        <v>10</v>
+      <c r="O26" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OFlaherty_2001_Cr.sbml</t>
+          <t>Hu.sbml</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OFlaherty2001_Cr_Human</t>
+          <t>Hu2023_BPA_Human</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Hu</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty%202001_Pb/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
+          <t>./models/oral/Bisphenols/Hu/summary.md</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>7</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>19</v>
+      </c>
+      <c r="K27" t="n">
         <v>6</v>
       </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>12</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>30</v>
-      </c>
       <c r="L27" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="M27" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="N27" t="n">
-        <v>1</v>
+        <v>65</v>
+      </c>
+      <c r="O27" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb.sbml</t>
+          <t>Loizou.sbml</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb_Human_Male</t>
+          <t>Loizou2022_BPA_Human</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Loizou</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Tebby_Pb/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>3</v>
+          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+        </is>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K28" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="L28" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="M28" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="N28" t="n">
-        <v>6</v>
+        <v>104</v>
+      </c>
+      <c r="O28" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg.sbml</t>
+          <t>Karrer.sbml</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg_Human</t>
+          <t>Karrer2018_BPA_Human</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Karrer</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Carrier_Hg/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>GI;Liver;Blood</t>
-        </is>
-      </c>
-      <c r="G29" t="n">
-        <v>3</v>
+          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+        </is>
       </c>
       <c r="H29" t="n">
+        <v>7</v>
+      </c>
+      <c r="I29" t="n">
         <v>0</v>
       </c>
-      <c r="I29" t="n">
-        <v>3</v>
-      </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="K29" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="M29" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>63</v>
+      </c>
+      <c r="O29" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>KjellstromCd.sbml</t>
+          <t>Christensen.sbml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Kjellstrom1978_Cd_Human</t>
+          <t>Christensen2013_BPA_Human</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Christensen</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Kjellstrom_Cd/summary.md</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
-        </is>
-      </c>
-      <c r="G30" t="n">
-        <v>9</v>
+          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Stomach;Blood;Bladder</t>
+        </is>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I30" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="L30" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="M30" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N30" t="n">
-        <v>11</v>
+        <v>28</v>
+      </c>
+      <c r="O30" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Karrer.sbml</t>
+          <t>Gilbert_Sandoval.sbml</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Karrer2018_BPA_Human</t>
+          <t>GilbertSandoval</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Gilbert_Sandoval</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
-        </is>
-      </c>
-      <c r="G31" t="n">
-        <v>7</v>
+          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
+        </is>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I31" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K31" t="n">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="L31" t="n">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="M31" t="n">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="N31" t="n">
-        <v>28</v>
+        <v>40</v>
+      </c>
+      <c r="O31" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Sharma.sbml</t>
+          <t>Mendez_Catala.sbml</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sharma2018_BPA_Human</t>
+          <t>Mandez_Catal_2021_Human_PBK</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Mendez_Catala</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
-        </is>
-      </c>
-      <c r="G32" t="n">
-        <v>5</v>
+          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
+        </is>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I32" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="K32" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="L32" t="n">
-        <v>5</v>
+        <v>87</v>
       </c>
       <c r="M32" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="N32" t="n">
-        <v>9</v>
+        <v>59</v>
+      </c>
+      <c r="O32" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hu.sbml</t>
+          <t>Notenboom.sbml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hu2023_BPA_Human</t>
+          <t>Notenboom2023_DON_Human</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Notenboom</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Hu/summary.md</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>7</v>
+          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Lumen;Liver;Blood;Rest</t>
+        </is>
       </c>
       <c r="H33" t="n">
+        <v>4</v>
+      </c>
+      <c r="I33" t="n">
         <v>0</v>
-      </c>
-      <c r="I33" t="n">
-        <v>19</v>
       </c>
       <c r="J33" t="n">
         <v>6</v>
       </c>
       <c r="K33" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="M33" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="N33" t="n">
-        <v>27</v>
+        <v>3</v>
+      </c>
+      <c r="O33" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Christensen.sbml</t>
+          <t>Mukherjee.sbml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Christensen2013_BPA_Human</t>
+          <t>Mukherjee2014_Human_PBK</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Mukherjee</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Stomach;Blood;Bladder</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>3</v>
+          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
+        </is>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J34" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="K34" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L34" t="n">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="M34" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="N34" t="n">
-        <v>6</v>
+        <v>30</v>
+      </c>
+      <c r="O34" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Moreau.sbml</t>
+          <t>Wang.sbml</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Moreau2025_BPA_Human</t>
+          <t>Wang2023_DON_Human</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Wang</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
+          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>8</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>9</v>
+      </c>
+      <c r="K35" t="n">
+        <v>5</v>
+      </c>
+      <c r="L35" t="n">
+        <v>48</v>
+      </c>
+      <c r="M35" t="n">
+        <v>17</v>
+      </c>
+      <c r="N35" t="n">
         <v>7</v>
       </c>
-      <c r="H35" t="n">
-        <v>1</v>
-      </c>
-      <c r="I35" t="n">
-        <v>9</v>
-      </c>
-      <c r="J35" t="n">
-        <v>3</v>
-      </c>
-      <c r="K35" t="n">
-        <v>37</v>
-      </c>
-      <c r="L35" t="n">
-        <v>37</v>
-      </c>
-      <c r="M35" t="n">
-        <v>75</v>
-      </c>
-      <c r="N35" t="n">
-        <v>28</v>
+      <c r="O35" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>OFlaherty2001.sbml</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Deepika2022_BPA_Human</t>
+          <t>OFlaherty2001_Cr_Human</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>OFlaherty 2001</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>5</v>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
+        </is>
       </c>
       <c r="H36" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I36" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="K36" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="M36" t="n">
-        <v>76</v>
+        <v>12</v>
       </c>
       <c r="N36" t="n">
-        <v>29</v>
+        <v>19</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Shin.sbml</t>
+          <t>KjellstromNordberg1978.sbml</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Shin2004_BPA_Human</t>
+          <t>KjellstromNordberg1978_Cd_Human</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>KjellstromNordberg 1978</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Shin/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>7</v>
+          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+        </is>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I37" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J37" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K37" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="L37" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="M37" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="N37" t="n">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="O37" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mielke.sbml</t>
+          <t>Tebby2022.sbml</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mielke2009_BPA_Human</t>
+          <t>Tebby2022_Pb_Human</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Tebby 2022</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>4</v>
+          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Liver;Blood;Rest</t>
+        </is>
       </c>
       <c r="H38" t="n">
+        <v>3</v>
+      </c>
+      <c r="I38" t="n">
         <v>0</v>
       </c>
-      <c r="I38" t="n">
-        <v>6</v>
-      </c>
       <c r="J38" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" t="n">
         <v>0</v>
       </c>
-      <c r="K38" t="n">
-        <v>22</v>
-      </c>
       <c r="L38" t="n">
+        <v>21</v>
+      </c>
+      <c r="M38" t="n">
         <v>2</v>
       </c>
-      <c r="M38" t="n">
-        <v>9</v>
-      </c>
       <c r="N38" t="n">
+        <v>5</v>
+      </c>
+      <c r="O38" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Teeguarden.sbml</t>
+          <t>ElMasri2008.sbml</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Teeguarden2005_BPA_Human</t>
+          <t>ElMasri2008_As_Human</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>ElMasri 2008</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>GILumen;Liver;Blood;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>5</v>
+          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
+        </is>
       </c>
       <c r="H39" t="n">
+        <v>8</v>
+      </c>
+      <c r="I39" t="n">
         <v>0</v>
       </c>
-      <c r="I39" t="n">
-        <v>8</v>
-      </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="K39" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="L39" t="n">
-        <v>6</v>
+        <v>78</v>
       </c>
       <c r="M39" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="N39" t="n">
-        <v>9</v>
+        <v>107</v>
+      </c>
+      <c r="O39" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Yang.sbml</t>
+          <t>Carrier2001.sbml</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yang2015_BPA_Human</t>
+          <t>Carrier2001_Hg_Human</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Carrier 2001</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Yang/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>7</v>
+          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>GI;Liver;Blood</t>
+        </is>
       </c>
       <c r="H40" t="n">
+        <v>3</v>
+      </c>
+      <c r="I40" t="n">
         <v>0</v>
       </c>
-      <c r="I40" t="n">
-        <v>19</v>
-      </c>
       <c r="J40" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="M40" t="n">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="N40" t="n">
-        <v>29</v>
+        <v>1</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Loizou.sbml</t>
+          <t>Ruiz2010_Male.sbml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Loizou2022_BPA_Human</t>
+          <t>Ruiz2010_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Ruiz 2010_Female</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>5</v>
+          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+        </is>
       </c>
       <c r="H41" t="n">
+        <v>9</v>
+      </c>
+      <c r="I41" t="n">
         <v>2</v>
       </c>
-      <c r="I41" t="n">
-        <v>8</v>
-      </c>
       <c r="J41" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K41" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="L41" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="M41" t="n">
-        <v>104</v>
+        <v>13</v>
       </c>
       <c r="N41" t="n">
-        <v>33</v>
+        <v>10</v>
+      </c>
+      <c r="O41" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Husoy.sbml</t>
+          <t>Ruiz2010_Female.sbml</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Husoy2024_PFOA_Human</t>
+          <t>Ruiz2010_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Ruiz 2010_Female</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Husoy/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>5</v>
+          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+        </is>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I42" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K42" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="L42" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="M42" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="N42" t="n">
-        <v>3</v>
+        <v>10</v>
+      </c>
+      <c r="O42" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Clewell1999.sbml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Chen2022_PFOS_Human</t>
+          <t>Clewell_Hg_Human</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Clewell 1999</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Chen/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>6</v>
+          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+        </is>
       </c>
       <c r="H43" t="n">
+        <v>7</v>
+      </c>
+      <c r="I43" t="n">
         <v>0</v>
       </c>
-      <c r="I43" t="n">
-        <v>6</v>
-      </c>
       <c r="J43" t="n">
+        <v>9</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1</v>
+      </c>
+      <c r="L43" t="n">
+        <v>42</v>
+      </c>
+      <c r="M43" t="n">
+        <v>14</v>
+      </c>
+      <c r="N43" t="n">
+        <v>20</v>
+      </c>
+      <c r="O43" t="n">
         <v>2</v>
-      </c>
-      <c r="K43" t="n">
-        <v>29</v>
-      </c>
-      <c r="L43" t="n">
-        <v>7</v>
-      </c>
-      <c r="M43" t="n">
-        <v>10</v>
-      </c>
-      <c r="N43" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LoccisanoPFOA.sbml</t>
+          <t>Pouillot2022.sbml</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Loccisano2011_PFOA_Human</t>
+          <t>Pouillot2022_Cd_Human</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Pouillot 2022</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Loccisano_PFOA/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>4</v>
+          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+        </is>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K44" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="M44" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="N44" t="n">
-        <v>3</v>
+        <v>7</v>
+      </c>
+      <c r="O44" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Ou2018.sbml</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Deepika2021_PFOS_Human</t>
+          <t>Ou2018_Hg_Human</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Ou 2018</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Deepika/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
+          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>7</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>9</v>
+      </c>
+      <c r="K45" t="n">
+        <v>2</v>
+      </c>
+      <c r="L45" t="n">
+        <v>42</v>
+      </c>
+      <c r="M45" t="n">
+        <v>14</v>
+      </c>
+      <c r="N45" t="n">
+        <v>23</v>
+      </c>
+      <c r="O45" t="n">
         <v>4</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" t="n">
-        <v>4</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>25</v>
-      </c>
-      <c r="L45" t="n">
-        <v>1</v>
-      </c>
-      <c r="M45" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LoccisanoPFOS.sbml</t>
+          <t>Bechaux2014_Male.sbml</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Loccisano2011_PFOS_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Loccisano_PFOS/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>4</v>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+        </is>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K46" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="L46" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="M46" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="N46" t="n">
-        <v>3</v>
+        <v>9</v>
+      </c>
+      <c r="O46" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ChouLin.sbml</t>
+          <t>Bechaux2014_Female.sbml</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Chou_Lin2021_PFOS_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>6</v>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+        </is>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I47" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J47" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K47" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="L47" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="M47" t="n">
+        <v>12</v>
+      </c>
+      <c r="N47" t="n">
+        <v>9</v>
+      </c>
+      <c r="O47" t="n">
         <v>10</v>
-      </c>
-      <c r="N47" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Worley.sbml</t>
+          <t>OFlaherty2000.sbml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Worley2017_PFOA_Human</t>
+          <t>OFlaherty2000_Pb_Human</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>OFlaherty 2000</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Worley/summary.md</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
+          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Liver;Blood;Rest</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>3</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>21</v>
+      </c>
+      <c r="M48" t="n">
+        <v>3</v>
+      </c>
+      <c r="N48" t="n">
+        <v>3</v>
+      </c>
+      <c r="O48" t="n">
         <v>6</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" t="n">
-        <v>6</v>
-      </c>
-      <c r="J48" t="n">
-        <v>2</v>
-      </c>
-      <c r="K48" t="n">
-        <v>29</v>
-      </c>
-      <c r="L48" t="n">
-        <v>7</v>
-      </c>
-      <c r="M48" t="n">
-        <v>10</v>
-      </c>
-      <c r="N48" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>model_C_inh_exh_art_ven.sbml</t>
+          <t>model_A_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>inhalation_C_art_ven</t>
+          <t>inhalation_A_art_ven</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>model_A_inh_exh_art_ven</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>inhalation</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Structure_C_alveolar_lung</t>
-        </is>
-      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>./models/inhalation/Structure_C_alveolar_lung/summary.md</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung;Bloodlung</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>6</v>
+          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Air;Arterial;Venous;RestofBody</t>
+        </is>
       </c>
       <c r="H49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I49" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K49" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="L49" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="M49" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="N49" t="n">
-        <v>20</v>
+        <v>14</v>
+      </c>
+      <c r="O49" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven.sbml</t>
+          <t>model_C_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>inhalation_B_art_ven</t>
+          <t>inhalation_C_art_ven</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
+          <t>model_C_inh_exh_art_ven</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
           <t>inhalation</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Structure_B_lung</t>
-        </is>
-      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>./models/inhalation/Structure_B_lung/summary.md</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>5</v>
+          <t>./models/inhalation/Generic/Structure_C_alveolar_lung/summary.md</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Air;Arterial;Venous;RestofBody;Lung;Bloodlung</t>
+        </is>
       </c>
       <c r="H50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I50" t="n">
         <v>5</v>
       </c>
       <c r="J50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K50" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="L50" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="M50" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="N50" t="n">
-        <v>16</v>
+        <v>22</v>
+      </c>
+      <c r="O50" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>model_A_inh_exh_art_ven.sbml</t>
+          <t>model_B_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>inhalation_A_art_ven</t>
+          <t>inhalation_B_art_ven</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>model_B_inh_exh_art_ven</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
           <t>inhalation</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Structure_A_direct_blood</t>
-        </is>
-      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>./models/inhalation/Structure_A_direct_blood/summary.md</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>4</v>
+          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Air;Arterial;Venous;RestofBody;Lung</t>
+        </is>
       </c>
       <c r="H51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I51" t="n">
         <v>4</v>
       </c>
       <c r="J51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K51" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="L51" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="M51" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N51" t="n">
-        <v>12</v>
+        <v>18</v>
+      </c>
+      <c r="O51" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed c828160 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -548,10 +548,10 @@
         <v>7</v>
       </c>
       <c r="N2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -609,10 +609,10 @@
         <v>7</v>
       </c>
       <c r="N3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -792,10 +792,10 @@
         <v>7</v>
       </c>
       <c r="N6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Deployed 48a7763 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -496,17 +496,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Godin.sbml</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chen2022_PFOS_Human</t>
+          <t>Godin_Pyrethroid_Human</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Godin</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -516,58 +516,58 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Chen/summary.md</t>
+          <t>./models/oral/Pesticides/Godin/summary.md</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L2" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="M2" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="O2" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ChouLin.sbml</t>
+          <t>Zwartsen.sbml</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chou_Lin2021_PFOS_Human</t>
+          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ChouLin</t>
+          <t>Zwartsen</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -577,58 +577,58 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L3" t="n">
+        <v>57</v>
+      </c>
+      <c r="M3" t="n">
+        <v>57</v>
+      </c>
+      <c r="N3" t="n">
+        <v>114</v>
+      </c>
+      <c r="O3" t="n">
         <v>29</v>
-      </c>
-      <c r="M3" t="n">
-        <v>7</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Deepika2021_PFOS_Human</t>
+          <t>Wei_Permethrin_Human</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -638,58 +638,58 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Deepika/summary.md</t>
+          <t>./models/oral/Pesticides/Wei/summary.md</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J4" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L4" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="O4" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LoccisanoPFOA.sbml</t>
+          <t>Zhao.sbml</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Loccisano2011_PFOA_Human</t>
+          <t>Zhao2019_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LoccisanoPFOA</t>
+          <t>Zhao</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -699,58 +699,58 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Loccisano_PFOA/summary.md</t>
+          <t>./models/oral/Pesticides/Zhao/summary.md</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>4</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="O5" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Worley.sbml</t>
+          <t>Tonnelier.sbml</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Worley2017_PFOA_Human</t>
+          <t>Tonnelier2012_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Worley</t>
+          <t>Tonnelier</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -760,58 +760,58 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Worley/summary.md</t>
+          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J6" t="n">
         <v>6</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="M6" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="O6" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LoccisanoPFOS.sbml</t>
+          <t>Timchalk.sbml</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Loccisano2011_PFOS_Human</t>
+          <t>Timchalk2002_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LoccisanoPFOS</t>
+          <t>Timchalk</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -821,58 +821,58 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Loccisano_PFOS/summary.md</t>
+          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L7" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="M7" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="O7" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Husoy.sbml</t>
+          <t>Moreau_Carbaryl.sbml</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Husoy2024_PFOA_Human</t>
+          <t>Moreau_Deltamethrin_Human</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Husoy</t>
+          <t>Moreau_Deltamethrin</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -882,58 +882,58 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Husoy/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L8" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="M8" t="n">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="N8" t="n">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="O8" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tonnelier.sbml</t>
+          <t>Moreau_Deltamethrin.sbml</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tonnelier2012_Chlorpyrifos_Human</t>
+          <t>Moreau_Deltamethrin_Human</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tonnelier</t>
+          <t>Moreau_Deltamethrin</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -948,37 +948,37 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L9" t="n">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="M9" t="n">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="N9" t="n">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="O9" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10">
@@ -1045,17 +1045,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Zhao.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Zhao2019_Chlorpyrifos_Human</t>
+          <t>Bouchard2010_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Zhao</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1070,53 +1070,53 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zhao/summary.md</t>
+          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>Gut;Blood;Rest</t>
         </is>
       </c>
       <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" t="n">
         <v>4</v>
       </c>
-      <c r="I11" t="n">
+      <c r="K11" t="n">
         <v>4</v>
       </c>
-      <c r="J11" t="n">
-        <v>7</v>
-      </c>
-      <c r="K11" t="n">
-        <v>7</v>
-      </c>
       <c r="L11" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="M11" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="O11" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bouchard.sbml</t>
+          <t>Mallick.sbml</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bouchard2010_Chlorpyrifos_Human</t>
+          <t>Mallick2020_Pyrethroids_Human</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bouchard</t>
+          <t>Mallick</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1131,53 +1131,53 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
+          <t>./models/oral/Pesticides/Mallick/summary.md</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Gut;Blood;Rest</t>
+          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L12" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="M12" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="N12" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="O12" t="n">
-        <v>4</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Godin.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Godin_Pyrethroid_Human</t>
+          <t>Deepika2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Godin</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1187,58 +1187,58 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Godin/summary.md</t>
+          <t>./models/oral/PFAS/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="M13" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="N13" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Zwartsen.sbml</t>
+          <t>ChouLin.sbml</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
+          <t>Chou_Lin2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Zwartsen</t>
+          <t>ChouLin</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1248,58 +1248,58 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
+          <t>./models/oral/PFAS/ChouLin/summary.md</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" t="n">
+        <v>29</v>
+      </c>
+      <c r="M14" t="n">
         <v>7</v>
       </c>
-      <c r="K14" t="n">
-        <v>7</v>
-      </c>
-      <c r="L14" t="n">
-        <v>57</v>
-      </c>
-      <c r="M14" t="n">
-        <v>57</v>
-      </c>
       <c r="N14" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl.sbml</t>
+          <t>Worley.sbml</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin_Human</t>
+          <t>Worley2017_PFOA_Human</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin</t>
+          <t>Worley</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1309,58 +1309,58 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/PFAS/Worley/summary.md</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H15" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>6</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>29</v>
+      </c>
+      <c r="M15" t="n">
         <v>7</v>
       </c>
-      <c r="I15" t="n">
-        <v>7</v>
-      </c>
-      <c r="J15" t="n">
-        <v>9</v>
-      </c>
-      <c r="K15" t="n">
-        <v>9</v>
-      </c>
-      <c r="L15" t="n">
-        <v>37</v>
-      </c>
-      <c r="M15" t="n">
-        <v>37</v>
-      </c>
       <c r="N15" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin_Human</t>
+          <t>Chen2022_PFOS_Human</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1370,58 +1370,58 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/PFAS/Chen/summary.md</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" t="n">
+        <v>29</v>
+      </c>
+      <c r="M16" t="n">
         <v>7</v>
       </c>
-      <c r="I16" t="n">
-        <v>7</v>
-      </c>
-      <c r="J16" t="n">
-        <v>9</v>
-      </c>
-      <c r="K16" t="n">
-        <v>9</v>
-      </c>
-      <c r="L16" t="n">
-        <v>37</v>
-      </c>
-      <c r="M16" t="n">
-        <v>37</v>
-      </c>
       <c r="N16" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Timchalk.sbml</t>
+          <t>LoccisanoPFOS.sbml</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Timchalk2002_Chlorpyrifos_Human</t>
+          <t>Loccisano2011_PFOS_Human</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Timchalk</t>
+          <t>LoccisanoPFOS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1431,58 +1431,58 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+          <t>./models/oral/PFAS/Loccisano_PFOS/summary.md</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>25</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
         <v>3</v>
-      </c>
-      <c r="I17" t="n">
-        <v>3</v>
-      </c>
-      <c r="J17" t="n">
-        <v>5</v>
-      </c>
-      <c r="K17" t="n">
-        <v>5</v>
-      </c>
-      <c r="L17" t="n">
-        <v>23</v>
-      </c>
-      <c r="M17" t="n">
-        <v>23</v>
-      </c>
-      <c r="N17" t="n">
-        <v>46</v>
-      </c>
-      <c r="O17" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Wei.sbml</t>
+          <t>Husoy.sbml</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Wei_Permethrin_Human</t>
+          <t>Husoy2024_PFOA_Human</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>Husoy</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1492,58 +1492,58 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Wei/summary.md</t>
+          <t>./models/oral/PFAS/Husoy/summary.md</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
+          <t>GI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I18" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="K18" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="M18" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>104</v>
+        <v>2</v>
       </c>
       <c r="O18" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mallick.sbml</t>
+          <t>LoccisanoPFOA.sbml</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mallick2020_Pyrethroids_Human</t>
+          <t>Loccisano2011_PFOA_Human</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mallick</t>
+          <t>LoccisanoPFOA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1553,58 +1553,58 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Mallick/summary.md</t>
+          <t>./models/oral/PFAS/Loccisano_PFOA/summary.md</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K19" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="M19" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Teeguarden.sbml</t>
+          <t>ElMasri2008.sbml</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Teeguarden2005_BPA_Human</t>
+          <t>ElMasri2008_As_Human</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Teeguarden</t>
+          <t>ElMasri 2008</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1614,58 +1614,58 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>GILumen;Liver;Blood;Rest;Feces</t>
+          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L20" t="n">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="M20" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="N20" t="n">
-        <v>12</v>
+        <v>107</v>
       </c>
       <c r="O20" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Bechaux2014_Male.sbml</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Deepika2022_BPA_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1675,58 +1675,58 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J21" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="M21" t="n">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="N21" t="n">
-        <v>76</v>
+        <v>9</v>
       </c>
       <c r="O21" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sharma.sbml</t>
+          <t>Bechaux2014_Female.sbml</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sharma2018_BPA_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1736,58 +1736,58 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="M22" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="N22" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="O22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Shin.sbml</t>
+          <t>Tebby2022.sbml</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Shin2004_BPA_Human</t>
+          <t>Tebby2022_Pb_Human</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Shin</t>
+          <t>Tebby 2022</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1797,58 +1797,58 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Shin/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="M23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O23" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Yang.sbml</t>
+          <t>Carrier2001.sbml</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yang2015_BPA_Human</t>
+          <t>Carrier2001_Hg_Human</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Yang</t>
+          <t>Carrier 2001</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1858,58 +1858,58 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Yang/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>GI;Liver;Blood</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="M24" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="N24" t="n">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Moreau.sbml</t>
+          <t>Pouillot2022.sbml</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Moreau2025_BPA_Human</t>
+          <t>Pouillot2022_Cd_Human</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Moreau</t>
+          <t>Pouillot 2022</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1919,58 +1919,58 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J25" t="n">
         <v>9</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L25" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="M25" t="n">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="N25" t="n">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="O25" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mielke.sbml</t>
+          <t>KjellstromNordberg1978.sbml</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mielke2009_BPA_Human</t>
+          <t>KjellstromNordberg1978_Cd_Human</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mielke</t>
+          <t>KjellstromNordberg 1978</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1980,58 +1980,58 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="M26" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="N26" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O26" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hu.sbml</t>
+          <t>OFlaherty2001.sbml</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Hu2023_BPA_Human</t>
+          <t>OFlaherty2001_Cr_Human</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hu</t>
+          <t>OFlaherty 2001</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2041,58 +2041,58 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Hu/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
+        <v>12</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>30</v>
+      </c>
+      <c r="M27" t="n">
+        <v>12</v>
+      </c>
+      <c r="N27" t="n">
         <v>19</v>
       </c>
-      <c r="K27" t="n">
-        <v>6</v>
-      </c>
-      <c r="L27" t="n">
-        <v>60</v>
-      </c>
-      <c r="M27" t="n">
-        <v>27</v>
-      </c>
-      <c r="N27" t="n">
-        <v>65</v>
-      </c>
       <c r="O27" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Loizou.sbml</t>
+          <t>OFlaherty2000.sbml</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Loizou2022_BPA_Human</t>
+          <t>OFlaherty2000_Pb_Human</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Loizou</t>
+          <t>OFlaherty 2000</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2102,58 +2102,58 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="M28" t="n">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="N28" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="O28" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Karrer.sbml</t>
+          <t>Ou2018.sbml</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Karrer2018_BPA_Human</t>
+          <t>Ou2018_Hg_Human</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Karrer</t>
+          <t>Ou 2018</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2163,17 +2163,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -2183,38 +2183,38 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="K29" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="M29" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="N29" t="n">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="O29" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Christensen.sbml</t>
+          <t>Clewell1999.sbml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Christensen2013_BPA_Human</t>
+          <t>Clewell_Hg_Human</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Christensen</t>
+          <t>Clewell 1999</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2224,58 +2224,58 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Stomach;Blood;Bladder</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I30" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="M30" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="N30" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="O30" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval.sbml</t>
+          <t>Ruiz2010_Female.sbml</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GilbertSandoval</t>
+          <t>Ruiz2010_Cd_Human_Male</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval</t>
+          <t>Ruiz 2010_Male</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2285,58 +2285,58 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H31" t="n">
+        <v>9</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" t="n">
+        <v>9</v>
+      </c>
+      <c r="K31" t="n">
+        <v>2</v>
+      </c>
+      <c r="L31" t="n">
+        <v>15</v>
+      </c>
+      <c r="M31" t="n">
         <v>13</v>
       </c>
-      <c r="I31" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" t="n">
-        <v>15</v>
-      </c>
-      <c r="K31" t="n">
+      <c r="N31" t="n">
+        <v>10</v>
+      </c>
+      <c r="O31" t="n">
         <v>11</v>
-      </c>
-      <c r="L31" t="n">
-        <v>46</v>
-      </c>
-      <c r="M31" t="n">
-        <v>18</v>
-      </c>
-      <c r="N31" t="n">
-        <v>40</v>
-      </c>
-      <c r="O31" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mendez_Catala.sbml</t>
+          <t>Ruiz2010_Male.sbml</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Mandez_Catal_2021_Human_PBK</t>
+          <t>Ruiz2010_Cd_Human_Male</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Mendez_Catala</t>
+          <t>Ruiz 2010_Male</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2346,58 +2346,58 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J32" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="K32" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" t="n">
+        <v>15</v>
+      </c>
+      <c r="M32" t="n">
         <v>13</v>
       </c>
-      <c r="L32" t="n">
-        <v>87</v>
-      </c>
-      <c r="M32" t="n">
-        <v>29</v>
-      </c>
       <c r="N32" t="n">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="O32" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Notenboom.sbml</t>
+          <t>Yang.sbml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Notenboom2023_DON_Human</t>
+          <t>Yang2015_BPA_Human</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Notenboom</t>
+          <t>Yang</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2407,58 +2407,58 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
+          <t>./models/oral/Bisphenols/Yang/summary.md</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Lumen;Liver;Blood;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
+        <v>19</v>
+      </c>
+      <c r="K33" t="n">
+        <v>8</v>
+      </c>
+      <c r="L33" t="n">
+        <v>59</v>
+      </c>
+      <c r="M33" t="n">
+        <v>26</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
         <v>6</v>
-      </c>
-      <c r="K33" t="n">
-        <v>1</v>
-      </c>
-      <c r="L33" t="n">
-        <v>20</v>
-      </c>
-      <c r="M33" t="n">
-        <v>2</v>
-      </c>
-      <c r="N33" t="n">
-        <v>3</v>
-      </c>
-      <c r="O33" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mukherjee.sbml</t>
+          <t>Teeguarden.sbml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Mukherjee2014_Human_PBK</t>
+          <t>Teeguarden2005_BPA_Human</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Mukherjee</t>
+          <t>Teeguarden</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2468,58 +2468,58 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
+          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
+          <t>GILumen;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="K34" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="M34" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="N34" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Wang.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Wang2023_DON_Human</t>
+          <t>Deepika2022_BPA_Human</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Wang</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2529,58 +2529,58 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
+          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
         <v>8</v>
       </c>
-      <c r="I35" t="n">
+      <c r="K35" t="n">
         <v>1</v>
       </c>
-      <c r="J35" t="n">
-        <v>9</v>
-      </c>
-      <c r="K35" t="n">
+      <c r="L35" t="n">
+        <v>36</v>
+      </c>
+      <c r="M35" t="n">
         <v>5</v>
       </c>
-      <c r="L35" t="n">
-        <v>48</v>
-      </c>
-      <c r="M35" t="n">
-        <v>17</v>
-      </c>
       <c r="N35" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="O35" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OFlaherty2001.sbml</t>
+          <t>Sharma.sbml</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>OFlaherty2001_Cr_Human</t>
+          <t>Sharma2018_BPA_Human</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OFlaherty 2001</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2590,58 +2590,58 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
+          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H36" t="n">
+        <v>5</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>8</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="n">
+        <v>38</v>
+      </c>
+      <c r="M36" t="n">
         <v>6</v>
       </c>
-      <c r="I36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" t="n">
+      <c r="N36" t="n">
+        <v>20</v>
+      </c>
+      <c r="O36" t="n">
         <v>12</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" t="n">
-        <v>30</v>
-      </c>
-      <c r="M36" t="n">
-        <v>12</v>
-      </c>
-      <c r="N36" t="n">
-        <v>19</v>
-      </c>
-      <c r="O36" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978.sbml</t>
+          <t>Hu.sbml</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978_Cd_Human</t>
+          <t>Hu2023_BPA_Human</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KjellstromNordberg 1978</t>
+          <t>Hu</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2651,58 +2651,58 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
+          <t>./models/oral/Bisphenols/Hu/summary.md</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="K37" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L37" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="M37" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="N37" t="n">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="O37" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Tebby2022.sbml</t>
+          <t>Christensen.sbml</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb_Human</t>
+          <t>Christensen2013_BPA_Human</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Tebby 2022</t>
+          <t>Christensen</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2712,17 +2712,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
+          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Stomach;Blood;Bladder</t>
         </is>
       </c>
       <c r="H38" t="n">
@@ -2735,35 +2735,35 @@
         <v>3</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L38" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="M38" t="n">
+        <v>6</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
         <v>2</v>
-      </c>
-      <c r="N38" t="n">
-        <v>5</v>
-      </c>
-      <c r="O38" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ElMasri2008.sbml</t>
+          <t>Loizou.sbml</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ElMasri2008_As_Human</t>
+          <t>Loizou2022_BPA_Human</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ElMasri 2008</t>
+          <t>Loizou</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2773,58 +2773,58 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
+          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H39" t="n">
+        <v>5</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
         <v>8</v>
       </c>
-      <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="n">
+      <c r="K39" t="n">
+        <v>4</v>
+      </c>
+      <c r="L39" t="n">
+        <v>36</v>
+      </c>
+      <c r="M39" t="n">
+        <v>35</v>
+      </c>
+      <c r="N39" t="n">
+        <v>96</v>
+      </c>
+      <c r="O39" t="n">
         <v>32</v>
-      </c>
-      <c r="K39" t="n">
-        <v>2</v>
-      </c>
-      <c r="L39" t="n">
-        <v>78</v>
-      </c>
-      <c r="M39" t="n">
-        <v>16</v>
-      </c>
-      <c r="N39" t="n">
-        <v>107</v>
-      </c>
-      <c r="O39" t="n">
-        <v>19</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Carrier2001.sbml</t>
+          <t>Karrer.sbml</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg_Human</t>
+          <t>Karrer2018_BPA_Human</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Carrier 2001</t>
+          <t>Karrer</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2834,58 +2834,58 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
+          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>GI;Liver;Blood</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L40" t="n">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="M40" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="N40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O40" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ruiz2010_Male.sbml</t>
+          <t>Shin.sbml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>Shin2004_BPA_Human</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Female</t>
+          <t>Shin</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2895,58 +2895,58 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+          <t>./models/oral/Bisphenols/Shin/summary.md</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L41" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="M41" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="N41" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O41" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ruiz2010_Female.sbml</t>
+          <t>Moreau.sbml</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>Moreau2025_BPA_Human</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Female</t>
+          <t>Moreau</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2956,58 +2956,58 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
         <v>9</v>
       </c>
       <c r="K42" t="n">
+        <v>3</v>
+      </c>
+      <c r="L42" t="n">
+        <v>35</v>
+      </c>
+      <c r="M42" t="n">
+        <v>35</v>
+      </c>
+      <c r="N42" t="n">
         <v>2</v>
       </c>
-      <c r="L42" t="n">
-        <v>15</v>
-      </c>
-      <c r="M42" t="n">
-        <v>13</v>
-      </c>
-      <c r="N42" t="n">
-        <v>10</v>
-      </c>
       <c r="O42" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Clewell1999.sbml</t>
+          <t>Mielke.sbml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Clewell_Hg_Human</t>
+          <t>Mielke2009_BPA_Human</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Clewell 1999</t>
+          <t>Mielke</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3017,58 +3017,58 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
+          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="M43" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="N43" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="O43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Pouillot2022.sbml</t>
+          <t>Mendez_Catala.sbml</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Pouillot2022_Cd_Human</t>
+          <t>Mandez_Catal_2021_Human_PBK</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Pouillot 2022</t>
+          <t>Mendez_Catala</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3078,58 +3078,58 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K44" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="L44" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="M44" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="N44" t="n">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="O44" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ou2018.sbml</t>
+          <t>Notenboom.sbml</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ou2018_Hg_Human</t>
+          <t>Notenboom2023_DON_Human</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ou 2018</t>
+          <t>Notenboom</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3139,58 +3139,58 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
+          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>Lumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K45" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" t="n">
+        <v>20</v>
+      </c>
+      <c r="M45" t="n">
         <v>2</v>
       </c>
-      <c r="L45" t="n">
-        <v>42</v>
-      </c>
-      <c r="M45" t="n">
-        <v>14</v>
-      </c>
       <c r="N45" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="O45" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Bechaux2014_Male.sbml</t>
+          <t>Wang.sbml</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>Wang2023_DON_Human</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>Wang</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3200,58 +3200,58 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J46" t="n">
         <v>9</v>
       </c>
       <c r="K46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L46" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="M46" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="N46" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O46" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Bechaux2014_Female.sbml</t>
+          <t>Gilbert_Sandoval.sbml</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>GilbertSandoval</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>Gilbert_Sandoval</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3261,58 +3261,58 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H47" t="n">
+        <v>13</v>
+      </c>
+      <c r="I47" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" t="n">
+        <v>15</v>
+      </c>
+      <c r="K47" t="n">
+        <v>11</v>
+      </c>
+      <c r="L47" t="n">
+        <v>46</v>
+      </c>
+      <c r="M47" t="n">
+        <v>18</v>
+      </c>
+      <c r="N47" t="n">
+        <v>40</v>
+      </c>
+      <c r="O47" t="n">
         <v>9</v>
-      </c>
-      <c r="I47" t="n">
-        <v>3</v>
-      </c>
-      <c r="J47" t="n">
-        <v>9</v>
-      </c>
-      <c r="K47" t="n">
-        <v>3</v>
-      </c>
-      <c r="L47" t="n">
-        <v>15</v>
-      </c>
-      <c r="M47" t="n">
-        <v>12</v>
-      </c>
-      <c r="N47" t="n">
-        <v>9</v>
-      </c>
-      <c r="O47" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OFlaherty2000.sbml</t>
+          <t>Mukherjee.sbml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb_Human</t>
+          <t>Mukherjee2014_Human_PBK</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>OFlaherty 2000</t>
+          <t>Mukherjee</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3322,58 +3322,58 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J48" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L48" t="n">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="M48" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="N48" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="O48" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>model_A_inh_exh_art_ven.sbml</t>
+          <t>model_B_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>inhalation_A_art_ven</t>
+          <t>inhalation_B_art_ven</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>model_A_inh_exh_art_ven</t>
+          <t>model_B_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3388,37 +3388,37 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody</t>
+          <t>Air;Arterial;Venous;RestofBody;Lung</t>
         </is>
       </c>
       <c r="H49" t="n">
+        <v>5</v>
+      </c>
+      <c r="I49" t="n">
         <v>4</v>
       </c>
-      <c r="I49" t="n">
-        <v>3</v>
-      </c>
       <c r="J49" t="n">
+        <v>5</v>
+      </c>
+      <c r="K49" t="n">
         <v>4</v>
       </c>
-      <c r="K49" t="n">
-        <v>3</v>
-      </c>
       <c r="L49" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="M49" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N49" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="O49" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50">
@@ -3485,17 +3485,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven.sbml</t>
+          <t>model_A_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>inhalation_B_art_ven</t>
+          <t>inhalation_A_art_ven</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven</t>
+          <t>model_A_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3510,37 +3510,37 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung</t>
+          <t>Air;Arterial;Venous;RestofBody</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I51" t="n">
+        <v>3</v>
+      </c>
+      <c r="J51" t="n">
         <v>4</v>
       </c>
-      <c r="J51" t="n">
-        <v>5</v>
-      </c>
       <c r="K51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L51" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M51" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="N51" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="O51" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 0a96ab1 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1167,17 +1167,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Loccisano.sbml</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Deepika2021_PFOS_Human</t>
+          <t>Loccisano2011_PFAS_Human</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Loccisano</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Deepika/summary.md</t>
+          <t>./models/oral/PFAS/Loccisano/summary.md</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1228,17 +1228,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ChouLin.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Chou_Lin2021_PFOS_Human</t>
+          <t>Deepika2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ChouLin</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1253,31 +1253,31 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+          <t>./models/oral/PFAS/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="M14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -1289,17 +1289,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Worley.sbml</t>
+          <t>ChouLin.sbml</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Worley2017_PFOA_Human</t>
+          <t>Chou_Lin2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Worley</t>
+          <t>ChouLin</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Worley/summary.md</t>
+          <t>./models/oral/PFAS/ChouLin/summary.md</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1350,17 +1350,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Worley.sbml</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Chen2022_PFOS_Human</t>
+          <t>Worley2017_PFOA_Human</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Worley</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Chen/summary.md</t>
+          <t>./models/oral/PFAS/Worley/summary.md</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1411,17 +1411,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LoccisanoPFOS.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Loccisano2011_PFOS_Human</t>
+          <t>Chen2022_PFOS_Human</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LoccisanoPFOS</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1436,31 +1436,31 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Loccisano_PFOS/summary.md</t>
+          <t>./models/oral/PFAS/Chen/summary.md</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L17" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="M17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N17" t="n">
         <v>0</v>
@@ -1533,17 +1533,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LoccisanoPFOA.sbml</t>
+          <t>ElMasri2008.sbml</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Loccisano2011_PFOA_Human</t>
+          <t>ElMasri2008_As_Human</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LoccisanoPFOA</t>
+          <t>ElMasri 2008</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1553,58 +1553,58 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Loccisano_PFOA/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L19" t="n">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="O19" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ElMasri2008.sbml</t>
+          <t>Bechaux2014_Male.sbml</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ElMasri2008_As_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ElMasri 2008</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1619,43 +1619,43 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J20" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>78</v>
+        <v>15</v>
       </c>
       <c r="M20" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="N20" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
       <c r="O20" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bechaux2014_Male.sbml</t>
+          <t>Bechaux2014_Female.sbml</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1716,17 +1716,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bechaux2014_Female.sbml</t>
+          <t>Tebby2022.sbml</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>Tebby2022_Pb_Human</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>Tebby 2022</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1741,53 +1741,53 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
         <v>3</v>
       </c>
-      <c r="J22" t="n">
-        <v>9</v>
-      </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="M22" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="N22" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O22" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Tebby2022.sbml</t>
+          <t>Carrier2001.sbml</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb_Human</t>
+          <t>Carrier2001_Hg_Human</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tebby 2022</t>
+          <t>Carrier 2001</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1802,12 +1802,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GI;Liver;Blood</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -1823,32 +1823,32 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="M23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Carrier2001.sbml</t>
+          <t>Pouillot2022.sbml</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg_Human</t>
+          <t>Pouillot2022_Cd_Human</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Carrier 2001</t>
+          <t>Pouillot 2022</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1863,53 +1863,53 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>GI;Liver;Blood</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L24" t="n">
+        <v>14</v>
+      </c>
+      <c r="M24" t="n">
         <v>12</v>
       </c>
-      <c r="M24" t="n">
-        <v>3</v>
-      </c>
       <c r="N24" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Pouillot2022.sbml</t>
+          <t>KjellstromNordberg1978.sbml</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pouillot2022_Cd_Human</t>
+          <t>KjellstromNordberg1978_Cd_Human</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pouillot 2022</t>
+          <t>KjellstromNordberg 1978</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1945,32 +1945,32 @@
         <v>2</v>
       </c>
       <c r="L25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N25" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="O25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978.sbml</t>
+          <t>OFlaherty2001.sbml</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978_Cd_Human</t>
+          <t>OFlaherty2001_Cr_Human</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>KjellstromNordberg 1978</t>
+          <t>OFlaherty 2001</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1985,53 +1985,53 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="M26" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N26" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="O26" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OFlaherty2001.sbml</t>
+          <t>OFlaherty2000.sbml</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OFlaherty2001_Cr_Human</t>
+          <t>OFlaherty2000_Pb_Human</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>OFlaherty 2001</t>
+          <t>OFlaherty 2000</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2046,53 +2046,53 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H27" t="n">
+        <v>3</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>21</v>
+      </c>
+      <c r="M27" t="n">
+        <v>3</v>
+      </c>
+      <c r="N27" t="n">
+        <v>3</v>
+      </c>
+      <c r="O27" t="n">
         <v>6</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="n">
-        <v>12</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
-        <v>30</v>
-      </c>
-      <c r="M27" t="n">
-        <v>12</v>
-      </c>
-      <c r="N27" t="n">
-        <v>19</v>
-      </c>
-      <c r="O27" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OFlaherty2000.sbml</t>
+          <t>Ou2018.sbml</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb_Human</t>
+          <t>Ou2018_Hg_Human</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>OFlaherty 2000</t>
+          <t>Ou 2018</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2107,53 +2107,53 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L28" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="M28" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="N28" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="O28" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ou2018.sbml</t>
+          <t>Clewell1999.sbml</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ou2018_Hg_Human</t>
+          <t>Clewell_Hg_Human</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ou 2018</t>
+          <t>Clewell 1999</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2186,7 +2186,7 @@
         <v>9</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
         <v>42</v>
@@ -2195,26 +2195,26 @@
         <v>14</v>
       </c>
       <c r="N29" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="O29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Clewell1999.sbml</t>
+          <t>Ruiz2010_Female.sbml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Clewell_Hg_Human</t>
+          <t>Ruiz2010_Cd_Human_Male</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Clewell 1999</t>
+          <t>Ruiz 2010_Male</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2229,43 +2229,43 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J30" t="n">
         <v>9</v>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L30" t="n">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="M30" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N30" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="O30" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ruiz2010_Female.sbml</t>
+          <t>Ruiz2010_Male.sbml</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2326,17 +2326,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ruiz2010_Male.sbml</t>
+          <t>Yang.sbml</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Male</t>
+          <t>Yang2015_BPA_Human</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Male</t>
+          <t>Yang</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2346,58 +2346,58 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+          <t>./models/oral/Bisphenols/Yang/summary.md</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L32" t="n">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="M32" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="N32" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Yang.sbml</t>
+          <t>Teeguarden.sbml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yang2015_BPA_Human</t>
+          <t>Teeguarden2005_BPA_Human</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Yang</t>
+          <t>Teeguarden</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2412,53 +2412,53 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Yang/summary.md</t>
+          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>GILumen;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="K33" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="M33" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="N33" t="n">
         <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Teeguarden.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Teeguarden2005_BPA_Human</t>
+          <t>Deepika2022_BPA_Human</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Teeguarden</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
+          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>GILumen;Liver;Blood;Rest;Feces</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -2494,32 +2494,32 @@
         <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M34" t="n">
+        <v>1</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="n">
         <v>6</v>
-      </c>
-      <c r="N34" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Sharma.sbml</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Deepika2022_BPA_Human</t>
+          <t>Sharma2018_BPA_Human</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
+          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2555,32 +2555,32 @@
         <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M35" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N35" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="O35" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Sharma.sbml</t>
+          <t>Hu.sbml</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Sharma2018_BPA_Human</t>
+          <t>Hu2023_BPA_Human</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>Hu</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2595,53 +2595,53 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
+          <t>./models/oral/Bisphenols/Hu/summary.md</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="K36" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L36" t="n">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="M36" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="N36" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="O36" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Hu.sbml</t>
+          <t>Christensen.sbml</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Hu2023_BPA_Human</t>
+          <t>Christensen2013_BPA_Human</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Hu</t>
+          <t>Christensen</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2656,53 +2656,53 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Hu/summary.md</t>
+          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Stomach;Blood;Bladder</t>
         </is>
       </c>
       <c r="H37" t="n">
+        <v>3</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" t="n">
+        <v>2</v>
+      </c>
+      <c r="L37" t="n">
         <v>7</v>
       </c>
-      <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="n">
-        <v>19</v>
-      </c>
-      <c r="K37" t="n">
+      <c r="M37" t="n">
         <v>6</v>
       </c>
-      <c r="L37" t="n">
-        <v>60</v>
-      </c>
-      <c r="M37" t="n">
-        <v>27</v>
-      </c>
       <c r="N37" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="O37" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Christensen.sbml</t>
+          <t>Loizou.sbml</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Christensen2013_BPA_Human</t>
+          <t>Loizou2022_BPA_Human</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Christensen</t>
+          <t>Loizou</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2717,53 +2717,53 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
+          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Stomach;Blood;Bladder</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L38" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="M38" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="N38" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="O38" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Loizou.sbml</t>
+          <t>Karrer.sbml</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Loizou2022_BPA_Human</t>
+          <t>Karrer2018_BPA_Human</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Loizou</t>
+          <t>Karrer</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2778,53 +2778,53 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
+          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K39" t="n">
         <v>4</v>
       </c>
       <c r="L39" t="n">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M39" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="N39" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="O39" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Karrer.sbml</t>
+          <t>Shin.sbml</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Karrer2018_BPA_Human</t>
+          <t>Shin2004_BPA_Human</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Karrer</t>
+          <t>Shin</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2839,12 +2839,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
+          <t>./models/oral/Bisphenols/Shin/summary.md</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -2854,38 +2854,38 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="K40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L40" t="n">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="M40" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>
       </c>
       <c r="O40" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Shin.sbml</t>
+          <t>Moreau.sbml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Shin2004_BPA_Human</t>
+          <t>Moreau2025_BPA_Human</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Shin</t>
+          <t>Moreau</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2900,53 +2900,53 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Shin/summary.md</t>
+          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H41" t="n">
         <v>7</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K41" t="n">
         <v>3</v>
       </c>
       <c r="L41" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="M41" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="N41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O41" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Moreau.sbml</t>
+          <t>Mielke.sbml</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Moreau2025_BPA_Human</t>
+          <t>Mielke2009_BPA_Human</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Moreau</t>
+          <t>Mielke</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2961,34 +2961,34 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
+          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="M42" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="N42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O42" t="n">
         <v>4</v>
@@ -2997,17 +2997,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mielke.sbml</t>
+          <t>Mendez_Catala.sbml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Mielke2009_BPA_Human</t>
+          <t>Mandez_Catal_2021_Human_PBK</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mielke</t>
+          <t>Mendez_Catala</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3017,58 +3017,58 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J43" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L43" t="n">
-        <v>22</v>
+        <v>87</v>
       </c>
       <c r="M43" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="O43" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mendez_Catala.sbml</t>
+          <t>Notenboom.sbml</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Mandez_Catal_2021_Human_PBK</t>
+          <t>Notenboom2023_DON_Human</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Mendez_Catala</t>
+          <t>Notenboom</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3083,53 +3083,53 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
+          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
+          <t>Lumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>6</v>
+      </c>
+      <c r="K44" t="n">
         <v>1</v>
       </c>
-      <c r="J44" t="n">
+      <c r="L44" t="n">
         <v>20</v>
       </c>
-      <c r="K44" t="n">
-        <v>13</v>
-      </c>
-      <c r="L44" t="n">
-        <v>87</v>
-      </c>
       <c r="M44" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="O44" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Notenboom.sbml</t>
+          <t>Wang.sbml</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Notenboom2023_DON_Human</t>
+          <t>Wang2023_DON_Human</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Notenboom</t>
+          <t>Wang</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3144,53 +3144,53 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
+          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Lumen;Liver;Blood;Rest</t>
+          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K45" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L45" t="n">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="M45" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="N45" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="O45" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Wang.sbml</t>
+          <t>Gilbert_Sandoval.sbml</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Wang2023_DON_Human</t>
+          <t>GilbertSandoval</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Wang</t>
+          <t>Gilbert_Sandoval</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3205,53 +3205,53 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
+          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I46" t="n">
         <v>1</v>
       </c>
       <c r="J46" t="n">
+        <v>15</v>
+      </c>
+      <c r="K46" t="n">
+        <v>11</v>
+      </c>
+      <c r="L46" t="n">
+        <v>46</v>
+      </c>
+      <c r="M46" t="n">
+        <v>18</v>
+      </c>
+      <c r="N46" t="n">
+        <v>40</v>
+      </c>
+      <c r="O46" t="n">
         <v>9</v>
-      </c>
-      <c r="K46" t="n">
-        <v>5</v>
-      </c>
-      <c r="L46" t="n">
-        <v>48</v>
-      </c>
-      <c r="M46" t="n">
-        <v>17</v>
-      </c>
-      <c r="N46" t="n">
-        <v>7</v>
-      </c>
-      <c r="O46" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval.sbml</t>
+          <t>Mukherjee.sbml</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GilbertSandoval</t>
+          <t>Mukherjee2014_Human_PBK</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval</t>
+          <t>Mukherjee</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3266,114 +3266,114 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
+          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J47" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K47" t="n">
         <v>11</v>
       </c>
       <c r="L47" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="M47" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N47" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O47" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mukherjee.sbml</t>
+          <t>model_B_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Mukherjee2014_Human_PBK</t>
+          <t>inhalation_B_art_ven</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mukherjee</t>
+          <t>model_B_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>inhalation</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
+          <t>Air;Arterial;Venous;RestofBody;Lung</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J48" t="n">
+        <v>5</v>
+      </c>
+      <c r="K48" t="n">
+        <v>4</v>
+      </c>
+      <c r="L48" t="n">
+        <v>18</v>
+      </c>
+      <c r="M48" t="n">
+        <v>17</v>
+      </c>
+      <c r="N48" t="n">
+        <v>18</v>
+      </c>
+      <c r="O48" t="n">
         <v>16</v>
-      </c>
-      <c r="K48" t="n">
-        <v>11</v>
-      </c>
-      <c r="L48" t="n">
-        <v>51</v>
-      </c>
-      <c r="M48" t="n">
-        <v>22</v>
-      </c>
-      <c r="N48" t="n">
-        <v>30</v>
-      </c>
-      <c r="O48" t="n">
-        <v>33</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven.sbml</t>
+          <t>model_C_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>inhalation_B_art_ven</t>
+          <t>inhalation_C_art_ven</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven</t>
+          <t>model_C_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3388,53 +3388,53 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_C_alveolar_lung/summary.md</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung</t>
+          <t>Air;Arterial;Venous;RestofBody;Lung;Bloodlung</t>
         </is>
       </c>
       <c r="H49" t="n">
+        <v>6</v>
+      </c>
+      <c r="I49" t="n">
         <v>5</v>
       </c>
-      <c r="I49" t="n">
-        <v>4</v>
-      </c>
       <c r="J49" t="n">
+        <v>6</v>
+      </c>
+      <c r="K49" t="n">
         <v>5</v>
       </c>
-      <c r="K49" t="n">
-        <v>4</v>
-      </c>
       <c r="L49" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="M49" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="N49" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="O49" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>model_C_inh_exh_art_ven.sbml</t>
+          <t>model_A_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>inhalation_C_art_ven</t>
+          <t>inhalation_A_art_ven</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>model_C_inh_exh_art_ven</t>
+          <t>model_A_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3449,97 +3449,36 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_C_alveolar_lung/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung;Bloodlung</t>
+          <t>Air;Arterial;Venous;RestofBody</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I50" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J50" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K50" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L50" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="M50" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="N50" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="O50" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>model_A_inh_exh_art_ven.sbml</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>inhalation_A_art_ven</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>model_A_inh_exh_art_ven</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>inhalation</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Air;Arterial;Venous;RestofBody</t>
-        </is>
-      </c>
-      <c r="H51" t="n">
-        <v>4</v>
-      </c>
-      <c r="I51" t="n">
-        <v>3</v>
-      </c>
-      <c r="J51" t="n">
-        <v>4</v>
-      </c>
-      <c r="K51" t="n">
-        <v>3</v>
-      </c>
-      <c r="L51" t="n">
-        <v>14</v>
-      </c>
-      <c r="M51" t="n">
-        <v>13</v>
-      </c>
-      <c r="N51" t="n">
-        <v>14</v>
-      </c>
-      <c r="O51" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 090ad8d with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,220 +496,220 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Godin.sbml</t>
+          <t>model_C_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Godin_Pyrethroid_Human</t>
+          <t>inhalation_C_art_ven</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Godin</t>
+          <t>model_C_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>inhalation</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Godin/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_C_alveolar_lung/summary.md</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
+          <t>Air;Arterial;Venous;RestofBody;Lung;Bloodlung</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L2" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="M2" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="N2" t="n">
-        <v>106</v>
+        <v>22</v>
       </c>
       <c r="O2" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zwartsen.sbml</t>
+          <t>model_B_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
+          <t>inhalation_B_art_ven</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Zwartsen</t>
+          <t>model_B_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>inhalation</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
+          <t>Air;Arterial;Venous;RestofBody;Lung</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>5</v>
       </c>
       <c r="I3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" t="n">
         <v>5</v>
       </c>
-      <c r="J3" t="n">
-        <v>7</v>
-      </c>
       <c r="K3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L3" t="n">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="M3" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="N3" t="n">
-        <v>114</v>
+        <v>18</v>
       </c>
       <c r="O3" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wei.sbml</t>
+          <t>model_A_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Wei_Permethrin_Human</t>
+          <t>inhalation_A_art_ven</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>model_A_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>inhalation</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Wei/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
+          <t>Air;Arterial;Venous;RestofBody</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="L4" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="M4" t="n">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="N4" t="n">
-        <v>104</v>
+        <v>14</v>
       </c>
       <c r="O4" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zhao.sbml</t>
+          <t>dermal-simple-model-Karrer-based.sbml</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Zhao2019_Chlorpyrifos_Human</t>
+          <t>BPA_Dermal_Simplified_Karrer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Zhao</t>
+          <t>dermal-simple-model-Karrer-based</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>dermal-simple-model-Karrer-based</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zhao/summary.md</t>
+          <t>./models/dermal/dermal-simple-model-Karrer-based/summary.md</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>SurfaceDepot;Skin;Plasma;Restbody</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -719,10 +719,10 @@
         <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L5" t="n">
         <v>26</v>
@@ -731,290 +731,290 @@
         <v>26</v>
       </c>
       <c r="N5" t="n">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tonnelier.sbml</t>
+          <t>Dermal_APM_CarrierBrunet1999_DermalOnly.sbml</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tonnelier2012_Chlorpyrifos_Human</t>
+          <t>Dermal_APM_CarrierBrunet1999_DermalOnly</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tonnelier</t>
+          <t>Dermal_APM_CarrierBrunet 1999_DermalOnly</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Dermal_APM_CarrierBrunet1999_DermalOnly</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
+          <t>./models/dermal/Dermal_APM_CarrierBrunet1999_DermalOnly/summary.md</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
+          <t>Skin;RestBody;Urine;NonObservedExcr</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" t="n">
         <v>6</v>
       </c>
-      <c r="K6" t="n">
+      <c r="M6" t="n">
         <v>6</v>
       </c>
-      <c r="L6" t="n">
-        <v>17</v>
-      </c>
-      <c r="M6" t="n">
-        <v>17</v>
-      </c>
       <c r="N6" t="n">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="O6" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Timchalk.sbml</t>
+          <t>dermal-simple-Quindroit-based.sbml</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Timchalk2002_Chlorpyrifos_Human</t>
+          <t>Dermal_PBK_Quindroit_Simplified</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Timchalk</t>
+          <t>dermal-simple-Quindroit-based</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>dermal-simple-Quindroit-based</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+          <t>./models/dermal/dermal-simple-Quindroit-based/summary.md</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>default_compartment;SkinSurface;StratumCorneum;Skin;ArterialBlood;VenousBlood;RestOfBody</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L7" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="M7" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="N7" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="O7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl.sbml</t>
+          <t>dermal-simple-Tonnelier-based.sbml</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin_Human</t>
+          <t>Dermal_PBK_Tonnelier_Simplified</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin</t>
+          <t>dermal-simple-Tonnelier-based</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>dermal-simple-Tonnelier-based</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/dermal/dermal-simple-Tonnelier-based/summary.md</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Skin;Blood;Liver</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" t="n">
         <v>9</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
         <v>9</v>
       </c>
-      <c r="L8" t="n">
-        <v>37</v>
-      </c>
-      <c r="M8" t="n">
-        <v>37</v>
-      </c>
       <c r="N8" t="n">
-        <v>108</v>
+        <v>32</v>
       </c>
       <c r="O8" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin.sbml</t>
+          <t>dermal-simple-Timchalk-based.sbml</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin_Human</t>
+          <t>Dermal_CPF_Timchalk2002_Simplified</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin</t>
+          <t>dermal-simple-Timchalk-based</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>dermal-simple-Timchalk-based</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/dermal/dermal-simple-Timchalk-based/summary.md</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Skin;ArterialBlood;VenousBlood;RestOfBody;Elimination</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I9" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K9" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="M9" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="N9" t="n">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>dermal-simple-Tornero-Velez-based.sbml</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chen_Fenitrothion_Human</t>
+          <t>permethrin_dermal_minPBK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>dermal-simple-Tornero-Velez-based</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>dermal-simple-Tornero-Velez-based</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Chen/summary.md</t>
+          <t>./models/dermal/dermal-simple-Tornero-Velez-based/summary.md</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
+          <t>default_compartment;Blood;RestBody;SC;VE</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -1024,58 +1024,58 @@
         <v>5</v>
       </c>
       <c r="J10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="M10" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="N10" t="n">
-        <v>88</v>
+        <v>38</v>
       </c>
       <c r="O10" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bouchard.sbml</t>
+          <t>dermal-steady-state-Dancik-based.sbml</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bouchard2010_Chlorpyrifos_Human</t>
+          <t>Dermal_Diffusion_Dancik2013</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bouchard</t>
+          <t>dermal-steady-state-Dancik-based</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>dermal-steady-state-Dancik-based</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
+          <t>./models/dermal/dermal-steady-state-Dancik-based/summary.md</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Gut;Blood;Rest</t>
+          <t>Stratum_Corneum;Viable_Epidermis;Dermis</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -1085,99 +1085,99 @@
         <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="M11" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="N11" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="O11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mallick.sbml</t>
+          <t>BPA_Dermal_simple-Hu-based.sbml</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mallick2020_Pyrethroids_Human</t>
+          <t>BPA_Dermal_PBK_Hu_layered</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mallick</t>
+          <t>BPA_Dermal_simple-Hu-based</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>BPA_Dermal_simple-Hu-based</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Mallick/summary.md</t>
+          <t>./models/dermal/BPA_Dermal_simple-Hu-based/summary.md</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
+          <t>SurfaceDepot;ExposedVE;Follicle;UnexposedSkin;Plasma;Restbody</t>
         </is>
       </c>
       <c r="H12" t="n">
         <v>6</v>
       </c>
       <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
         <v>6</v>
       </c>
-      <c r="J12" t="n">
-        <v>7</v>
-      </c>
       <c r="K12" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L12" t="n">
-        <v>36</v>
+        <v>67</v>
       </c>
       <c r="M12" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="N12" t="n">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="O12" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Loccisano.sbml</t>
+          <t>Mukherjee.sbml</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Loccisano2011_PFAS_Human</t>
+          <t>Mukherjee2014_Human_PBK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Loccisano</t>
+          <t>Mukherjee</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1187,58 +1187,58 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Loccisano/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L13" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="O13" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Mendez_Catala.sbml</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Deepika2021_PFOS_Human</t>
+          <t>Mandez_Catal_2021_Human_PBK</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Mendez_Catala</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1248,58 +1248,58 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Deepika/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L14" t="n">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="O14" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ChouLin.sbml</t>
+          <t>Gilbert_Sandoval.sbml</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Chou_Lin2021_PFOS_Human</t>
+          <t>GilbertSandoval</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ChouLin</t>
+          <t>Gilbert_Sandoval</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1309,58 +1309,58 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K15" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="L15" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="M15" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Worley.sbml</t>
+          <t>Notenboom.sbml</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Worley2017_PFOA_Human</t>
+          <t>Notenboom2023_DON_Human</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Worley</t>
+          <t>Notenboom</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1370,21 +1370,21 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Worley/summary.md</t>
+          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Lumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -1393,35 +1393,35 @@
         <v>6</v>
       </c>
       <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>20</v>
+      </c>
+      <c r="M16" t="n">
         <v>2</v>
       </c>
-      <c r="L16" t="n">
-        <v>29</v>
-      </c>
-      <c r="M16" t="n">
-        <v>7</v>
-      </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Wang.sbml</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chen2022_PFOS_Human</t>
+          <t>Wang2023_DON_Human</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Wang</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1431,58 +1431,58 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Chen/summary.md</t>
+          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L17" t="n">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="M17" t="n">
+        <v>17</v>
+      </c>
+      <c r="N17" t="n">
         <v>7</v>
       </c>
-      <c r="N17" t="n">
-        <v>0</v>
-      </c>
       <c r="O17" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Husoy.sbml</t>
+          <t>Shin.sbml</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Husoy2024_PFOA_Human</t>
+          <t>Shin2004_BPA_Human</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Husoy</t>
+          <t>Shin</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1492,58 +1492,58 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Husoy/summary.md</t>
+          <t>./models/oral/Bisphenols/Shin/summary.md</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L18" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ElMasri2008.sbml</t>
+          <t>Mielke.sbml</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ElMasri2008_As_Human</t>
+          <t>Mielke2009_BPA_Human</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ElMasri 2008</t>
+          <t>Mielke</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1553,58 +1553,58 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
+          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>22</v>
+      </c>
+      <c r="M19" t="n">
         <v>2</v>
       </c>
-      <c r="L19" t="n">
-        <v>78</v>
-      </c>
-      <c r="M19" t="n">
-        <v>16</v>
-      </c>
       <c r="N19" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bechaux2014_Male.sbml</t>
+          <t>Moreau.sbml</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>Moreau2025_BPA_Human</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>Moreau</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1614,24 +1614,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
         <v>9</v>
@@ -1640,32 +1640,32 @@
         <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="M20" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="N20" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="O20" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bechaux2014_Female.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>Deepika2022_BPA_Human</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1675,58 +1675,58 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="M21" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O21" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Tebby2022.sbml</t>
+          <t>Loizou.sbml</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb_Human</t>
+          <t>Loizou2022_BPA_Human</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tebby 2022</t>
+          <t>Loizou</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1736,58 +1736,58 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
+          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L22" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="M22" t="n">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="N22" t="n">
-        <v>5</v>
+        <v>96</v>
       </c>
       <c r="O22" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Carrier2001.sbml</t>
+          <t>Christensen.sbml</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg_Human</t>
+          <t>Christensen2013_BPA_Human</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Carrier 2001</t>
+          <t>Christensen</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1797,17 +1797,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
+          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>GI;Liver;Blood</t>
+          <t>Stomach;Blood;Bladder</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -1820,35 +1820,35 @@
         <v>3</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pouillot2022.sbml</t>
+          <t>Teeguarden.sbml</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pouillot2022_Cd_Human</t>
+          <t>Teeguarden2005_BPA_Human</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pouillot 2022</t>
+          <t>Teeguarden</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1858,58 +1858,58 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
+          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>GILumen;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="M24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="N24" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978.sbml</t>
+          <t>Hu.sbml</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978_Cd_Human</t>
+          <t>Hu2023_BPA_Human</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KjellstromNordberg 1978</t>
+          <t>Hu</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1919,58 +1919,58 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
+          <t>./models/oral/Bisphenols/Hu/summary.md</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="K25" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L25" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="M25" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="N25" t="n">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="O25" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>OFlaherty2001.sbml</t>
+          <t>Yang.sbml</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>OFlaherty2001_Cr_Human</t>
+          <t>Yang2015_BPA_Human</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>OFlaherty 2001</t>
+          <t>Yang</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1980,58 +1980,58 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
+          <t>./models/oral/Bisphenols/Yang/summary.md</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H26" t="n">
+        <v>7</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>18</v>
+      </c>
+      <c r="K26" t="n">
+        <v>8</v>
+      </c>
+      <c r="L26" t="n">
+        <v>59</v>
+      </c>
+      <c r="M26" t="n">
+        <v>26</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
         <v>6</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="n">
-        <v>12</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="n">
-        <v>30</v>
-      </c>
-      <c r="M26" t="n">
-        <v>12</v>
-      </c>
-      <c r="N26" t="n">
-        <v>19</v>
-      </c>
-      <c r="O26" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OFlaherty2000.sbml</t>
+          <t>Sharma.sbml</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb_Human</t>
+          <t>Sharma2018_BPA_Human</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>OFlaherty 2000</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2041,58 +2041,58 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
+          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="M27" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N27" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="O27" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ou2018.sbml</t>
+          <t>Karrer.sbml</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ou2018_Hg_Human</t>
+          <t>Karrer2018_BPA_Human</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ou 2018</t>
+          <t>Karrer</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2102,17 +2102,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
+          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -2122,38 +2122,38 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L28" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="M28" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="N28" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Clewell1999.sbml</t>
+          <t>ElMasri2008.sbml</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Clewell_Hg_Human</t>
+          <t>ElMasri2008_As_Human</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Clewell 1999</t>
+          <t>ElMasri 2008</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2168,53 +2168,53 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="K29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="M29" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="N29" t="n">
-        <v>20</v>
+        <v>107</v>
       </c>
       <c r="O29" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ruiz2010_Female.sbml</t>
+          <t>Ruiz2010_Male.sbml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Male</t>
+          <t>Ruiz2010_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Male</t>
+          <t>Ruiz 2010_Female</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2265,17 +2265,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ruiz2010_Male.sbml</t>
+          <t>Ruiz2010_Female.sbml</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Male</t>
+          <t>Ruiz2010_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Male</t>
+          <t>Ruiz 2010_Female</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2326,17 +2326,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Yang.sbml</t>
+          <t>Pouillot2022.sbml</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yang2015_BPA_Human</t>
+          <t>Pouillot2022_Cd_Human</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Yang</t>
+          <t>Pouillot 2022</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2346,58 +2346,58 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Yang/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H32" t="n">
+        <v>9</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" t="n">
+        <v>9</v>
+      </c>
+      <c r="K32" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" t="n">
+        <v>14</v>
+      </c>
+      <c r="M32" t="n">
+        <v>12</v>
+      </c>
+      <c r="N32" t="n">
         <v>7</v>
       </c>
-      <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="n">
-        <v>18</v>
-      </c>
-      <c r="K32" t="n">
-        <v>8</v>
-      </c>
-      <c r="L32" t="n">
-        <v>59</v>
-      </c>
-      <c r="M32" t="n">
-        <v>26</v>
-      </c>
-      <c r="N32" t="n">
-        <v>0</v>
-      </c>
       <c r="O32" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Teeguarden.sbml</t>
+          <t>Bechaux2014_Male.sbml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Teeguarden2005_BPA_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Teeguarden</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2407,58 +2407,58 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>GILumen;Liver;Blood;Rest;Feces</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="M33" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="N33" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="O33" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Bechaux2014_Female.sbml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Deepika2022_BPA_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2468,58 +2468,58 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J34" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="O34" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sharma.sbml</t>
+          <t>OFlaherty2000.sbml</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Sharma2018_BPA_Human</t>
+          <t>OFlaherty2000_Pb_Human</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>OFlaherty 2000</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2529,58 +2529,58 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="M35" t="n">
+        <v>3</v>
+      </c>
+      <c r="N35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O35" t="n">
         <v>6</v>
-      </c>
-      <c r="N35" t="n">
-        <v>20</v>
-      </c>
-      <c r="O35" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Hu.sbml</t>
+          <t>OFlaherty2001.sbml</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hu2023_BPA_Human</t>
+          <t>OFlaherty2001_Cr_Human</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hu</t>
+          <t>OFlaherty 2001</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2590,58 +2590,58 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Hu/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
+        <v>12</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>30</v>
+      </c>
+      <c r="M36" t="n">
+        <v>12</v>
+      </c>
+      <c r="N36" t="n">
         <v>19</v>
       </c>
-      <c r="K36" t="n">
-        <v>6</v>
-      </c>
-      <c r="L36" t="n">
-        <v>60</v>
-      </c>
-      <c r="M36" t="n">
-        <v>27</v>
-      </c>
-      <c r="N36" t="n">
-        <v>68</v>
-      </c>
       <c r="O36" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Christensen.sbml</t>
+          <t>Ou2018.sbml</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Christensen2013_BPA_Human</t>
+          <t>Ou2018_Hg_Human</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Christensen</t>
+          <t>Ou 2018</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2651,58 +2651,58 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Stomach;Blood;Bladder</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K37" t="n">
         <v>2</v>
       </c>
       <c r="L37" t="n">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="M37" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="N37" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="O37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Loizou.sbml</t>
+          <t>KjellstromNordberg1978.sbml</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Loizou2022_BPA_Human</t>
+          <t>KjellstromNordberg1978_Cd_Human</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Loizou</t>
+          <t>KjellstromNordberg 1978</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2712,58 +2712,58 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J38" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L38" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="M38" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="N38" t="n">
-        <v>96</v>
+        <v>10</v>
       </c>
       <c r="O38" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Karrer.sbml</t>
+          <t>Carrier2001.sbml</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Karrer2018_BPA_Human</t>
+          <t>Carrier2001_Hg_Human</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Karrer</t>
+          <t>Carrier 2001</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2773,58 +2773,58 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>GI;Liver;Blood</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="K39" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="M39" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="N39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O39" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Shin.sbml</t>
+          <t>Tebby2022.sbml</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Shin2004_BPA_Human</t>
+          <t>Tebby2022_Pb_Human</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Shin</t>
+          <t>Tebby 2022</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2834,58 +2834,58 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Shin/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="M40" t="n">
+        <v>2</v>
+      </c>
+      <c r="N40" t="n">
+        <v>5</v>
+      </c>
+      <c r="O40" t="n">
         <v>6</v>
-      </c>
-      <c r="N40" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Moreau.sbml</t>
+          <t>Clewell1999.sbml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Moreau2025_BPA_Human</t>
+          <t>Clewell_Hg_Human</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Moreau</t>
+          <t>Clewell 1999</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2895,58 +2895,58 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H41" t="n">
         <v>7</v>
       </c>
       <c r="I41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
         <v>9</v>
       </c>
       <c r="K41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="M41" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="N41" t="n">
+        <v>20</v>
+      </c>
+      <c r="O41" t="n">
         <v>2</v>
-      </c>
-      <c r="O41" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mielke.sbml</t>
+          <t>Tonnelier.sbml</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mielke2009_BPA_Human</t>
+          <t>Tonnelier2012_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Mielke</t>
+          <t>Tonnelier</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2956,58 +2956,58 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
+          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J42" t="n">
         <v>6</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L42" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="M42" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="O42" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mendez_Catala.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Mandez_Catal_2021_Human_PBK</t>
+          <t>Chen_Fenitrothion_Human</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mendez_Catala</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3017,58 +3017,58 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
+          <t>./models/oral/Pesticides/Chen/summary.md</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
+          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I43" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J43" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="K43" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="L43" t="n">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="M43" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="N43" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="O43" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Notenboom.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Notenboom2023_DON_Human</t>
+          <t>Wei_Permethrin_Human</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Notenboom</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3078,58 +3078,58 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
+          <t>./models/oral/Pesticides/Wei/summary.md</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Lumen;Liver;Blood;Rest</t>
+          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J44" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K44" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="L44" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="M44" t="n">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="N44" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="O44" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Wang.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Wang2023_DON_Human</t>
+          <t>Bouchard2010_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Wang</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3139,58 +3139,58 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
+          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
+          <t>Gut;Blood;Rest</t>
         </is>
       </c>
       <c r="H45" t="n">
+        <v>3</v>
+      </c>
+      <c r="I45" t="n">
+        <v>3</v>
+      </c>
+      <c r="J45" t="n">
+        <v>4</v>
+      </c>
+      <c r="K45" t="n">
+        <v>4</v>
+      </c>
+      <c r="L45" t="n">
+        <v>4</v>
+      </c>
+      <c r="M45" t="n">
+        <v>4</v>
+      </c>
+      <c r="N45" t="n">
         <v>8</v>
       </c>
-      <c r="I45" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" t="n">
-        <v>9</v>
-      </c>
-      <c r="K45" t="n">
-        <v>5</v>
-      </c>
-      <c r="L45" t="n">
-        <v>48</v>
-      </c>
-      <c r="M45" t="n">
-        <v>17</v>
-      </c>
-      <c r="N45" t="n">
-        <v>7</v>
-      </c>
       <c r="O45" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval.sbml</t>
+          <t>Moreau_Deltamethrin.sbml</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GilbertSandoval</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3200,58 +3200,58 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="I46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J46" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="K46" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L46" t="n">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="M46" t="n">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="N46" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
       <c r="O46" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Mukherjee.sbml</t>
+          <t>Moreau_Carbaryl.sbml</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Mukherjee2014_Human_PBK</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mukherjee</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3261,39 +3261,39 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I47" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J47" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="K47" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L47" t="n">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="M47" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="N47" t="n">
-        <v>30</v>
+        <v>108</v>
       </c>
       <c r="O47" t="n">
         <v>33</v>
@@ -3302,184 +3302,672 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven.sbml</t>
+          <t>Mallick.sbml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>inhalation_B_art_ven</t>
+          <t>Mallick2020_Pyrethroids_Human</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven</t>
+          <t>Mallick</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>inhalation</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
+          <t>./models/oral/Pesticides/Mallick/summary.md</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung</t>
+          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I48" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J48" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K48" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L48" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="M48" t="n">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="N48" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="O48" t="n">
-        <v>16</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>model_C_inh_exh_art_ven.sbml</t>
+          <t>Zhao.sbml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>inhalation_C_art_ven</t>
+          <t>Zhao2019_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>model_C_inh_exh_art_ven</t>
+          <t>Zhao</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>inhalation</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_C_alveolar_lung/summary.md</t>
+          <t>./models/oral/Pesticides/Zhao/summary.md</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung;Bloodlung</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J49" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K49" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L49" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="M49" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="N49" t="n">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="O49" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>model_A_inh_exh_art_ven.sbml</t>
+          <t>Zwartsen.sbml</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>inhalation_A_art_ven</t>
+          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>model_A_inh_exh_art_ven</t>
+          <t>Zwartsen</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>inhalation</t>
+          <t>oral</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
+          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody</t>
+          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H50" t="n">
+        <v>5</v>
+      </c>
+      <c r="I50" t="n">
+        <v>5</v>
+      </c>
+      <c r="J50" t="n">
+        <v>7</v>
+      </c>
+      <c r="K50" t="n">
+        <v>7</v>
+      </c>
+      <c r="L50" t="n">
+        <v>57</v>
+      </c>
+      <c r="M50" t="n">
+        <v>57</v>
+      </c>
+      <c r="N50" t="n">
+        <v>114</v>
+      </c>
+      <c r="O50" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Godin.sbml</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Godin_Pyrethroid_Human</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Godin</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Pesticides</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>./models/oral/Pesticides/Godin/summary.md</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>8</v>
+      </c>
+      <c r="I51" t="n">
+        <v>8</v>
+      </c>
+      <c r="J51" t="n">
+        <v>10</v>
+      </c>
+      <c r="K51" t="n">
+        <v>10</v>
+      </c>
+      <c r="L51" t="n">
+        <v>34</v>
+      </c>
+      <c r="M51" t="n">
+        <v>34</v>
+      </c>
+      <c r="N51" t="n">
+        <v>106</v>
+      </c>
+      <c r="O51" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Timchalk.sbml</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Timchalk2002_Chlorpyrifos_Human</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Timchalk</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Pesticides</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Liver;Blood;Rest</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>3</v>
+      </c>
+      <c r="I52" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" t="n">
+        <v>5</v>
+      </c>
+      <c r="K52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L52" t="n">
+        <v>23</v>
+      </c>
+      <c r="M52" t="n">
+        <v>23</v>
+      </c>
+      <c r="N52" t="n">
+        <v>46</v>
+      </c>
+      <c r="O52" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Chen.sbml</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Chen2022_PFOS_Human</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/Chen/summary.md</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>6</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
+        <v>6</v>
+      </c>
+      <c r="K53" t="n">
+        <v>2</v>
+      </c>
+      <c r="L53" t="n">
+        <v>29</v>
+      </c>
+      <c r="M53" t="n">
+        <v>7</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ChouLin.sbml</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Chou_Lin2021_PFOS_Human</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ChouLin</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>6</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>6</v>
+      </c>
+      <c r="K54" t="n">
+        <v>2</v>
+      </c>
+      <c r="L54" t="n">
+        <v>29</v>
+      </c>
+      <c r="M54" t="n">
+        <v>7</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Husoy.sbml</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Husoy2024_PFOA_Human</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Husoy</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/Husoy/summary.md</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>5</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>5</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="n">
+        <v>29</v>
+      </c>
+      <c r="M55" t="n">
+        <v>3</v>
+      </c>
+      <c r="N55" t="n">
+        <v>2</v>
+      </c>
+      <c r="O55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Worley.sbml</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Worley2017_PFOA_Human</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Worley</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/Worley/summary.md</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>6</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>6</v>
+      </c>
+      <c r="K56" t="n">
+        <v>2</v>
+      </c>
+      <c r="L56" t="n">
+        <v>29</v>
+      </c>
+      <c r="M56" t="n">
+        <v>7</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Deepika.sbml</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Deepika2021_PFOS_Human</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Deepika</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/Deepika/summary.md</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
         <v>4</v>
       </c>
-      <c r="I50" t="n">
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>4</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="n">
+        <v>25</v>
+      </c>
+      <c r="M57" t="n">
+        <v>1</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" t="n">
         <v>3</v>
       </c>
-      <c r="J50" t="n">
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Loccisano.sbml</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Loccisano2011_PFAS_Human</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Loccisano</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/Loccisano/summary.md</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
         <v>4</v>
       </c>
-      <c r="K50" t="n">
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>4</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="n">
+        <v>25</v>
+      </c>
+      <c r="M58" t="n">
+        <v>1</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="n">
         <v>3</v>
-      </c>
-      <c r="L50" t="n">
-        <v>14</v>
-      </c>
-      <c r="M50" t="n">
-        <v>13</v>
-      </c>
-      <c r="N50" t="n">
-        <v>14</v>
-      </c>
-      <c r="O50" t="n">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 0082779 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,17 +679,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>dermal-simple-model-Karrer-based.sbml</t>
+          <t>BPA_Dermal_simple-Hu-based.sbml</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BPA_Dermal_Simplified_Karrer</t>
+          <t>BPA_Dermal_PBK_Hu_layered</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>dermal-simple-model-Karrer-based</t>
+          <t>BPA_Dermal_simple-Hu-based</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -699,58 +699,58 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>dermal-simple-model-Karrer-based</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>./models/dermal/dermal-simple-model-Karrer-based/summary.md</t>
+          <t>./models/dermal/Bisphenols/Hu/summary.md</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SurfaceDepot;Skin;Plasma;Restbody</t>
+          <t>SurfaceDepot;ExposedVE;Follicle;UnexposedSkin;Plasma;Restbody;Urine</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K5" t="n">
         <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="M5" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="O5" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dermal_APM_CarrierBrunet1999_DermalOnly.sbml</t>
+          <t>dermal-simple-model-Karrer-based.sbml</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dermal_APM_CarrierBrunet1999_DermalOnly</t>
+          <t>BPA_Dermal_Simplified_Karrer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dermal_APM_CarrierBrunet 1999_DermalOnly</t>
+          <t>dermal-simple-model-Karrer-based</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -760,58 +760,58 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dermal_APM_CarrierBrunet1999_DermalOnly</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>./models/dermal/Dermal_APM_CarrierBrunet1999_DermalOnly/summary.md</t>
+          <t>./models/dermal/Bisphenols/Karrer/summary.md</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Skin;RestBody;Urine;NonObservedExcr</t>
+          <t>SurfaceDepot;Skin;Plasma;Restbody;Urine</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="M6" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="N6" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="O6" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dermal-simple-Quindroit-based.sbml</t>
+          <t>dermal-simple-Tonnelier-based.sbml</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dermal_PBK_Quindroit_Simplified</t>
+          <t>Dermal_PBK_Tonnelier_Simplified</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>dermal-simple-Quindroit-based</t>
+          <t>dermal-simple-Tonnelier-based</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -821,58 +821,58 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>dermal-simple-Quindroit-based</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>./models/dermal/dermal-simple-Quindroit-based/summary.md</t>
+          <t>./models/dermal/Pesticides/Tonnelier/summary.md</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>default_compartment;SkinSurface;StratumCorneum;Skin;ArterialBlood;VenousBlood;RestOfBody</t>
+          <t>DermalAbsorptionCompartment;PortalVeinBlood;Liver;SystemicCompartment;RenalExcretion</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L7" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="M7" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="N7" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dermal-simple-Tonnelier-based.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dermal_PBK_Tonnelier_Simplified</t>
+          <t>Dermal_PBK_Wei_Simplified</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>dermal-simple-Tonnelier-based</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -882,58 +882,58 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>dermal-simple-Tonnelier-based</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>./models/dermal/dermal-simple-Tonnelier-based/summary.md</t>
+          <t>./models/dermal/Pesticides/Wei/summary.md</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Skin;Blood;Liver</t>
+          <t>default_compartment;Skin;Blood;RestOfBody;UrinaryExcretion</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L8" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="M8" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="N8" t="n">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="O8" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dermal-simple-Timchalk-based.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dermal_CPF_Timchalk2002_Simplified</t>
+          <t>Bouchard2005_DermalOnly_Simplified</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>dermal-simple-Timchalk-based</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -943,58 +943,58 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>dermal-simple-Timchalk-based</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>./models/dermal/dermal-simple-Timchalk-based/summary.md</t>
+          <t>./models/dermal/Pesticides/Bouchard/summary.md</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Skin;ArterialBlood;VenousBlood;RestOfBody;Elimination</t>
+          <t>SkinSurf;Blood;RestOfBody;Urine</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="O9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dermal-simple-Tornero-Velez-based.sbml</t>
+          <t>dermal-simple-Quindroit-based.sbml</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>permethrin_dermal_minPBK</t>
+          <t>Dermal_PBK_Quindroit_Simplified</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>dermal-simple-Tornero-Velez-based</t>
+          <t>dermal-simple-Quindroit-based</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1004,58 +1004,58 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>dermal-simple-Tornero-Velez-based</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>./models/dermal/dermal-simple-Tornero-Velez-based/summary.md</t>
+          <t>./models/dermal/Pesticides/Quindroit/summary.md</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>default_compartment;Blood;RestBody;SC;VE</t>
+          <t>SkinSurface;StratumCorneum;Skin;ArterialBlood;VenousBlood;UrinaryTrack;RestOfBody</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="N10" t="n">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="O10" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dermal-steady-state-Dancik-based.sbml</t>
+          <t>Dermal_APM_CarrierBrunet1999_DermalOnly.sbml</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dermal_Diffusion_Dancik2013</t>
+          <t>Dermal_APM_CarrierBrunet1999_DermalOnly</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>dermal-steady-state-Dancik-based</t>
+          <t>Dermal_APM_CarrierBrunet 1999_DermalOnly</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1065,58 +1065,58 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>dermal-steady-state-Dancik-based</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>./models/dermal/dermal-steady-state-Dancik-based/summary.md</t>
+          <t>./models/dermal/Pesticides/Carrier_Brunet/summary.md</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Stratum_Corneum;Viable_Epidermis;Dermis</t>
+          <t>Skin;RestBody;Urine;NonObservedExcr</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L11" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="M11" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="O11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BPA_Dermal_simple-Hu-based.sbml</t>
+          <t>dermal-simple-Tornero-Velez-based.sbml</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BPA_Dermal_PBK_Hu_layered</t>
+          <t>permethrin_dermal_minPBK</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BPA_Dermal_simple-Hu-based</t>
+          <t>dermal-simple-Tornero-Velez-based</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1126,302 +1126,302 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BPA_Dermal_simple-Hu-based</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>./models/dermal/BPA_Dermal_simple-Hu-based/summary.md</t>
+          <t>./models/dermal/Pesticides/Tornero-Velez/summary.md</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SurfaceDepot;ExposedVE;Follicle;UnexposedSkin;Plasma;Restbody</t>
+          <t>SkinSurface;StratumCorneum;ViableEpidermis;ArterialBlood;VenousBlood;UrinaryExcretion;RestOfBody</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L12" t="n">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="M12" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="N12" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="O12" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mukherjee.sbml</t>
+          <t>Poet.sbml</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mukherjee2014_Human_PBK</t>
+          <t>Poet2014_DermalOnly_SimplifiedCPF</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mukherjee</t>
+          <t>Poet</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
+          <t>./models/dermal/Pesticides/Poet/summary.md</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
+          <t>Skin;ArterialBlood;VenousBlood;RestOfBody;Elimination</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J13" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="K13" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="L13" t="n">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="M13" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="N13" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="O13" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mendez_Catala.sbml</t>
+          <t>dermal-simple-Timchalk-based.sbml</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mandez_Catal_2021_Human_PBK</t>
+          <t>Dermal_CPF_Timchalk2002_Simplified</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mendez_Catala</t>
+          <t>dermal-simple-Timchalk-based</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
+          <t>./models/dermal/Pesticides/Timchalk/summary.md</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
+          <t>Skin;ArterialBlood;VenousBlood;RestOfBody;Elimination</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" t="n">
+        <v>27</v>
+      </c>
+      <c r="M14" t="n">
         <v>20</v>
       </c>
-      <c r="K14" t="n">
-        <v>13</v>
-      </c>
-      <c r="L14" t="n">
-        <v>87</v>
-      </c>
-      <c r="M14" t="n">
-        <v>29</v>
-      </c>
       <c r="N14" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="O14" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval.sbml</t>
+          <t>PFOA_dermal-simple-model-Husoy-based.sbml</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GilbertSandoval</t>
+          <t>Husoy2023_Dermal</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval</t>
+          <t>PFOA_dermal-simple-model-Husoy-based</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
+          <t>./models/dermal/PFAS/Husoy/summary.md</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
+          <t>Skin;Plasma;RestBody;Kidney;Urine</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="M15" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="N15" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="O15" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Notenboom.sbml</t>
+          <t>dermal-steady-state-Dancik-based.sbml</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Notenboom2023_DON_Human</t>
+          <t>Dermal_Diffusion_Dancik2013</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Notenboom</t>
+          <t>dermal-steady-state-Dancik-based</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>oral</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
+          <t>./models/dermal/Other/dermal-steady-state-Dancik-based/summary.md</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Lumen;Liver;Blood;Rest</t>
+          <t>Stratum_Corneum;Viable_Epidermis;Dermis</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J16" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" t="n">
+        <v>10</v>
+      </c>
+      <c r="M16" t="n">
+        <v>10</v>
+      </c>
+      <c r="N16" t="n">
+        <v>34</v>
+      </c>
+      <c r="O16" t="n">
         <v>6</v>
-      </c>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" t="n">
-        <v>20</v>
-      </c>
-      <c r="M16" t="n">
-        <v>2</v>
-      </c>
-      <c r="N16" t="n">
-        <v>3</v>
-      </c>
-      <c r="O16" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Wang.sbml</t>
+          <t>Mukherjee.sbml</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wang2023_DON_Human</t>
+          <t>Mukherjee2014_Human_PBK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wang</t>
+          <t>Mukherjee</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1436,53 +1436,53 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
+          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J17" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="K17" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="L17" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="M17" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N17" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="O17" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shin.sbml</t>
+          <t>Mendez_Catala.sbml</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shin2004_BPA_Human</t>
+          <t>Mandez_Catal_2021_Human_PBK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Shin</t>
+          <t>Mendez_Catala</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1492,58 +1492,58 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Shin/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="K18" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="L18" t="n">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="M18" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="O18" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mielke.sbml</t>
+          <t>Gilbert_Sandoval.sbml</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mielke2009_BPA_Human</t>
+          <t>GilbertSandoval</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mielke</t>
+          <t>Gilbert_Sandoval</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1553,58 +1553,58 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
+          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L19" t="n">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="M19" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O19" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Moreau.sbml</t>
+          <t>Notenboom.sbml</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Moreau2025_BPA_Human</t>
+          <t>Notenboom2023_DON_Human</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Moreau</t>
+          <t>Notenboom</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1614,58 +1614,58 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
+          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Lumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" t="n">
         <v>1</v>
       </c>
-      <c r="J20" t="n">
-        <v>9</v>
-      </c>
-      <c r="K20" t="n">
+      <c r="L20" t="n">
+        <v>20</v>
+      </c>
+      <c r="M20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" t="n">
         <v>3</v>
       </c>
-      <c r="L20" t="n">
-        <v>35</v>
-      </c>
-      <c r="M20" t="n">
-        <v>35</v>
-      </c>
-      <c r="N20" t="n">
-        <v>2</v>
-      </c>
       <c r="O20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Wang.sbml</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Deepika2022_BPA_Human</t>
+          <t>Wang2023_DON_Human</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Wang</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1675,58 +1675,58 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
+          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
         </is>
       </c>
       <c r="H21" t="n">
+        <v>8</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>9</v>
+      </c>
+      <c r="K21" t="n">
         <v>5</v>
       </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="n">
-        <v>8</v>
-      </c>
-      <c r="K21" t="n">
-        <v>1</v>
-      </c>
       <c r="L21" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O21" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Loizou.sbml</t>
+          <t>Shin.sbml</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Loizou2022_BPA_Human</t>
+          <t>Shin2004_BPA_Human</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Loizou</t>
+          <t>Shin</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1741,16 +1741,16 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
+          <t>./models/oral/Bisphenols/Shin/summary.md</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -1759,35 +1759,35 @@
         <v>8</v>
       </c>
       <c r="K22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="M22" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="N22" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="O22" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Christensen.sbml</t>
+          <t>Mielke.sbml</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Christensen2013_BPA_Human</t>
+          <t>Mielke2009_BPA_Human</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Christensen</t>
+          <t>Mielke</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1802,53 +1802,53 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
+          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Stomach;Blood;Bladder</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>22</v>
+      </c>
+      <c r="M23" t="n">
         <v>2</v>
       </c>
-      <c r="L23" t="n">
-        <v>7</v>
-      </c>
-      <c r="M23" t="n">
-        <v>6</v>
-      </c>
       <c r="N23" t="n">
         <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Teeguarden.sbml</t>
+          <t>Moreau.sbml</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Teeguarden2005_BPA_Human</t>
+          <t>Moreau2025_BPA_Human</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Teeguarden</t>
+          <t>Moreau</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1863,34 +1863,34 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
+          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>GILumen;Liver;Blood;Rest;Feces</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="M24" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O24" t="n">
         <v>4</v>
@@ -1899,17 +1899,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hu.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Hu2023_BPA_Human</t>
+          <t>Deepika2022_BPA_Human</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hu</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1924,53 +1924,53 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Hu/summary.md</t>
+          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="K25" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" t="n">
+        <v>28</v>
+      </c>
+      <c r="M25" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
         <v>6</v>
-      </c>
-      <c r="L25" t="n">
-        <v>60</v>
-      </c>
-      <c r="M25" t="n">
-        <v>27</v>
-      </c>
-      <c r="N25" t="n">
-        <v>68</v>
-      </c>
-      <c r="O25" t="n">
-        <v>27</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Yang.sbml</t>
+          <t>Loizou.sbml</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yang2015_BPA_Human</t>
+          <t>Loizou2022_BPA_Human</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Yang</t>
+          <t>Loizou</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1985,53 +1985,53 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Yang/summary.md</t>
+          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="K26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L26" t="n">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="M26" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="O26" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sharma.sbml</t>
+          <t>Christensen.sbml</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sharma2018_BPA_Human</t>
+          <t>Christensen2013_BPA_Human</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>Christensen</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2046,53 +2046,53 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
+          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Stomach;Blood;Bladder</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L27" t="n">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="M27" t="n">
         <v>6</v>
       </c>
       <c r="N27" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karrer.sbml</t>
+          <t>Teeguarden.sbml</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Karrer2018_BPA_Human</t>
+          <t>Teeguarden2005_BPA_Human</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Karrer</t>
+          <t>Teeguarden</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2107,53 +2107,53 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
+          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>GILumen;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="K28" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" t="n">
+        <v>30</v>
+      </c>
+      <c r="M28" t="n">
+        <v>6</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
         <v>4</v>
-      </c>
-      <c r="L28" t="n">
-        <v>59</v>
-      </c>
-      <c r="M28" t="n">
-        <v>26</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ElMasri2008.sbml</t>
+          <t>Hu.sbml</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ElMasri2008_As_Human</t>
+          <t>Hu2023_BPA_Human</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ElMasri 2008</t>
+          <t>Hu</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2163,58 +2163,58 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
+          <t>./models/oral/Bisphenols/Hu/summary.md</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L29" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="M29" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="N29" t="n">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="O29" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ruiz2010_Male.sbml</t>
+          <t>Yang.sbml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>Yang2015_BPA_Human</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Female</t>
+          <t>Yang</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2224,58 +2224,58 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+          <t>./models/oral/Bisphenols/Yang/summary.md</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="K30" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L30" t="n">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="M30" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="N30" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ruiz2010_Female.sbml</t>
+          <t>Sharma.sbml</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>Sharma2018_BPA_Human</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Female</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2285,58 +2285,58 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="M31" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="N31" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="O31" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pouillot2022.sbml</t>
+          <t>Karrer.sbml</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Pouillot2022_Cd_Human</t>
+          <t>Karrer2018_BPA_Human</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Pouillot 2022</t>
+          <t>Karrer</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2346,58 +2346,58 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
+          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L32" t="n">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="M32" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="N32" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Bechaux2014_Male.sbml</t>
+          <t>ElMasri2008.sbml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>ElMasri2008_As_Human</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>ElMasri 2008</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2412,53 +2412,53 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="M33" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="N33" t="n">
-        <v>9</v>
+        <v>107</v>
       </c>
       <c r="O33" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Bechaux2014_Female.sbml</t>
+          <t>Ruiz2010_Male.sbml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>Ruiz2010_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>Ruiz 2010_Female</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2485,41 +2485,41 @@
         <v>9</v>
       </c>
       <c r="I34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J34" t="n">
         <v>9</v>
       </c>
       <c r="K34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L34" t="n">
         <v>15</v>
       </c>
       <c r="M34" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N34" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O34" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OFlaherty2000.sbml</t>
+          <t>Ruiz2010_Female.sbml</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb_Human</t>
+          <t>Ruiz2010_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>OFlaherty 2000</t>
+          <t>Ruiz 2010_Female</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2534,53 +2534,53 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J35" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L35" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="M35" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="N35" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="O35" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OFlaherty2001.sbml</t>
+          <t>Pouillot2022.sbml</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>OFlaherty2001_Cr_Human</t>
+          <t>Pouillot2022_Cd_Human</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OFlaherty 2001</t>
+          <t>Pouillot 2022</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2595,53 +2595,53 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J36" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L36" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="M36" t="n">
         <v>12</v>
       </c>
       <c r="N36" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="O36" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ou2018.sbml</t>
+          <t>Bechaux2014_Male.sbml</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ou2018_Hg_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ou 2018</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2656,53 +2656,53 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J37" t="n">
         <v>9</v>
       </c>
       <c r="K37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="M37" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="N37" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="O37" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978.sbml</t>
+          <t>Bechaux2014_Female.sbml</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978_Cd_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>KjellstromNordberg 1978</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2729,41 +2729,41 @@
         <v>9</v>
       </c>
       <c r="I38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J38" t="n">
         <v>9</v>
       </c>
       <c r="K38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L38" t="n">
         <v>15</v>
       </c>
       <c r="M38" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N38" t="n">
+        <v>9</v>
+      </c>
+      <c r="O38" t="n">
         <v>10</v>
-      </c>
-      <c r="O38" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Carrier2001.sbml</t>
+          <t>OFlaherty2000.sbml</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg_Human</t>
+          <t>OFlaherty2000_Pb_Human</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Carrier 2001</t>
+          <t>OFlaherty 2000</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2778,12 +2778,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>GI;Liver;Blood</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H39" t="n">
@@ -2799,32 +2799,32 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="M39" t="n">
         <v>3</v>
       </c>
       <c r="N39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Tebby2022.sbml</t>
+          <t>OFlaherty2001.sbml</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb_Human</t>
+          <t>OFlaherty2001_Cr_Human</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Tebby 2022</t>
+          <t>OFlaherty 2001</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2839,53 +2839,53 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="M40" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="N40" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="O40" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Clewell1999.sbml</t>
+          <t>Ou2018.sbml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Clewell_Hg_Human</t>
+          <t>Ou2018_Hg_Human</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Clewell 1999</t>
+          <t>Ou 2018</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2918,7 +2918,7 @@
         <v>9</v>
       </c>
       <c r="K41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L41" t="n">
         <v>42</v>
@@ -2927,26 +2927,26 @@
         <v>14</v>
       </c>
       <c r="N41" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="O41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Tonnelier.sbml</t>
+          <t>KjellstromNordberg1978.sbml</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Tonnelier2012_Chlorpyrifos_Human</t>
+          <t>KjellstromNordberg1978_Cd_Human</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Tonnelier</t>
+          <t>KjellstromNordberg 1978</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2956,58 +2956,58 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I42" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K42" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L42" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M42" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="N42" t="n">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="O42" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Carrier2001.sbml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Chen_Fenitrothion_Human</t>
+          <t>Carrier2001_Hg_Human</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Carrier 2001</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3017,58 +3017,58 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Chen/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
+          <t>GI;Liver;Blood</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I43" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K43" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="M43" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="N43" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="O43" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Wei.sbml</t>
+          <t>Tebby2022.sbml</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Wei_Permethrin_Human</t>
+          <t>Tebby2022_Pb_Human</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>Tebby 2022</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3078,58 +3078,58 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Wei/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I44" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K44" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="M44" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
-        <v>104</v>
+        <v>5</v>
       </c>
       <c r="O44" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Bouchard.sbml</t>
+          <t>Clewell1999.sbml</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bouchard2010_Chlorpyrifos_Human</t>
+          <t>Clewell_Hg_Human</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bouchard</t>
+          <t>Clewell 1999</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3139,58 +3139,58 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Gut;Blood;Rest</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I45" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="M45" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="N45" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="O45" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin.sbml</t>
+          <t>Tonnelier.sbml</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>Tonnelier2012_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl</t>
+          <t>Tonnelier</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3205,53 +3205,53 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I46" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J46" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K46" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L46" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="M46" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="N46" t="n">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="O46" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>Chen_Fenitrothion_Human</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3266,53 +3266,53 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/Pesticides/Chen/summary.md</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H47" t="n">
+        <v>5</v>
+      </c>
+      <c r="I47" t="n">
+        <v>5</v>
+      </c>
+      <c r="J47" t="n">
         <v>7</v>
       </c>
-      <c r="I47" t="n">
+      <c r="K47" t="n">
         <v>7</v>
       </c>
-      <c r="J47" t="n">
-        <v>9</v>
-      </c>
-      <c r="K47" t="n">
-        <v>9</v>
-      </c>
       <c r="L47" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="M47" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="N47" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="O47" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mallick.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Mallick2020_Pyrethroids_Human</t>
+          <t>Wei_Permethrin_Human</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mallick</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3327,53 +3327,53 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Mallick/summary.md</t>
+          <t>./models/oral/Pesticides/Wei/summary.md</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
+          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I48" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J48" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K48" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L48" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="M48" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="N48" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="O48" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Zhao.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Zhao2019_Chlorpyrifos_Human</t>
+          <t>Bouchard2010_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Zhao</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3388,53 +3388,53 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zhao/summary.md</t>
+          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>Gut;Blood;Rest</t>
         </is>
       </c>
       <c r="H49" t="n">
+        <v>3</v>
+      </c>
+      <c r="I49" t="n">
+        <v>3</v>
+      </c>
+      <c r="J49" t="n">
         <v>4</v>
       </c>
-      <c r="I49" t="n">
+      <c r="K49" t="n">
         <v>4</v>
       </c>
-      <c r="J49" t="n">
-        <v>7</v>
-      </c>
-      <c r="K49" t="n">
-        <v>7</v>
-      </c>
       <c r="L49" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="M49" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="N49" t="n">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="O49" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Zwartsen.sbml</t>
+          <t>Moreau_Deltamethrin.sbml</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Zwartsen</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3449,53 +3449,53 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I50" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J50" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K50" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L50" t="n">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="M50" t="n">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="N50" t="n">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="O50" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Godin.sbml</t>
+          <t>Moreau_Carbaryl.sbml</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Godin_Pyrethroid_Human</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Godin</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3510,53 +3510,53 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Godin/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I51" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J51" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K51" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L51" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M51" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N51" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="O51" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Timchalk.sbml</t>
+          <t>Mallick.sbml</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Timchalk2002_Chlorpyrifos_Human</t>
+          <t>Mallick2020_Pyrethroids_Human</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Timchalk</t>
+          <t>Mallick</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3571,53 +3571,53 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+          <t>./models/oral/Pesticides/Mallick/summary.md</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I52" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J52" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K52" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L52" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="M52" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="N52" t="n">
-        <v>46</v>
+        <v>100</v>
       </c>
       <c r="O52" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Zhao.sbml</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Chen2022_PFOS_Human</t>
+          <t>Zhao2019_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Zhao</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3627,58 +3627,58 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Chen/summary.md</t>
+          <t>./models/oral/Pesticides/Zhao/summary.md</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J53" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K53" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L53" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="M53" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="N53" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="O53" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ChouLin.sbml</t>
+          <t>Zwartsen.sbml</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Chou_Lin2021_PFOS_Human</t>
+          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ChouLin</t>
+          <t>Zwartsen</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3688,58 +3688,58 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J54" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K54" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L54" t="n">
+        <v>57</v>
+      </c>
+      <c r="M54" t="n">
+        <v>57</v>
+      </c>
+      <c r="N54" t="n">
+        <v>114</v>
+      </c>
+      <c r="O54" t="n">
         <v>29</v>
-      </c>
-      <c r="M54" t="n">
-        <v>7</v>
-      </c>
-      <c r="N54" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Husoy.sbml</t>
+          <t>Godin.sbml</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Husoy2024_PFOA_Human</t>
+          <t>Godin_Pyrethroid_Human</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Husoy</t>
+          <t>Godin</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3749,58 +3749,58 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Husoy/summary.md</t>
+          <t>./models/oral/Pesticides/Godin/summary.md</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J55" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L55" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="M55" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="N55" t="n">
-        <v>2</v>
+        <v>106</v>
       </c>
       <c r="O55" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Worley.sbml</t>
+          <t>Timchalk.sbml</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Worley2017_PFOA_Human</t>
+          <t>Timchalk2002_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Worley</t>
+          <t>Timchalk</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3810,58 +3810,58 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Worley/summary.md</t>
+          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H56" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I56" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J56" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K56" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L56" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M56" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="N56" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="O56" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Deepika2021_PFOS_Human</t>
+          <t>Chen2022_PFOS_Human</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3876,31 +3876,31 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Deepika/summary.md</t>
+          <t>./models/oral/PFAS/Chen/summary.md</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L57" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="M57" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N57" t="n">
         <v>0</v>
@@ -3912,61 +3912,305 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>ChouLin.sbml</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Chou_Lin2021_PFOS_Human</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ChouLin</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>6</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>6</v>
+      </c>
+      <c r="K58" t="n">
+        <v>2</v>
+      </c>
+      <c r="L58" t="n">
+        <v>29</v>
+      </c>
+      <c r="M58" t="n">
+        <v>7</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Husoy.sbml</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Husoy2024_PFOA_Human</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Husoy</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/Husoy/summary.md</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>5</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="n">
+        <v>5</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="n">
+        <v>29</v>
+      </c>
+      <c r="M59" t="n">
+        <v>3</v>
+      </c>
+      <c r="N59" t="n">
+        <v>2</v>
+      </c>
+      <c r="O59" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Worley.sbml</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Worley2017_PFOA_Human</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Worley</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/Worley/summary.md</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>6</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="n">
+        <v>6</v>
+      </c>
+      <c r="K60" t="n">
+        <v>2</v>
+      </c>
+      <c r="L60" t="n">
+        <v>29</v>
+      </c>
+      <c r="M60" t="n">
+        <v>7</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Deepika.sbml</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Deepika2021_PFOS_Human</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Deepika</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>PFAS</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>./models/oral/PFAS/Deepika/summary.md</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>GI;Liver;Plasma;Rest</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>4</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="n">
+        <v>4</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="n">
+        <v>25</v>
+      </c>
+      <c r="M61" t="n">
+        <v>1</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>Loccisano.sbml</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>Loccisano2011_PFAS_Human</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>Loccisano</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>oral</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>oral</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>PFAS</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>./models/oral/PFAS/Loccisano/summary.md</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
-      <c r="H58" t="n">
+      <c r="H62" t="n">
         <v>4</v>
       </c>
-      <c r="I58" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" t="n">
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
         <v>4</v>
       </c>
-      <c r="K58" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" t="n">
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="n">
         <v>25</v>
       </c>
-      <c r="M58" t="n">
+      <c r="M62" t="n">
         <v>1</v>
       </c>
-      <c r="N58" t="n">
-        <v>0</v>
-      </c>
-      <c r="O58" t="n">
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 271258b with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,13 +722,13 @@
         <v>7</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
         <v>62</v>
       </c>
       <c r="M5" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="N5" t="n">
         <v>56</v>
@@ -1759,13 +1759,13 @@
         <v>8</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
         <v>28</v>
       </c>
       <c r="M22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N22" t="n">
         <v>0</v>
@@ -1826,7 +1826,7 @@
         <v>22</v>
       </c>
       <c r="M23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N23" t="n">
         <v>0</v>
@@ -1881,19 +1881,19 @@
         <v>9</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M24" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="N24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -1942,13 +1942,13 @@
         <v>8</v>
       </c>
       <c r="K25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
         <v>28</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
@@ -2003,19 +2003,19 @@
         <v>8</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
         <v>36</v>
       </c>
       <c r="M26" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -2064,13 +2064,13 @@
         <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L27" t="n">
         <v>7</v>
       </c>
       <c r="M27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
@@ -2122,10 +2122,10 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
         <v>30</v>
@@ -2143,17 +2143,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hu.sbml</t>
+          <t>Yang.sbml</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hu2023_BPA_Human</t>
+          <t>Yang2015_BPA_Human</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hu</t>
+          <t>Yang</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Hu/summary.md</t>
+          <t>./models/oral/Bisphenols/Yang/summary.md</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2183,38 +2183,38 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="K29" t="n">
+        <v>3</v>
+      </c>
+      <c r="L29" t="n">
+        <v>59</v>
+      </c>
+      <c r="M29" t="n">
+        <v>25</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
         <v>6</v>
-      </c>
-      <c r="L29" t="n">
-        <v>60</v>
-      </c>
-      <c r="M29" t="n">
-        <v>27</v>
-      </c>
-      <c r="N29" t="n">
-        <v>68</v>
-      </c>
-      <c r="O29" t="n">
-        <v>27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Yang.sbml</t>
+          <t>Sharma.sbml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yang2015_BPA_Human</t>
+          <t>Sharma2018_BPA_Human</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Yang</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2229,31 +2229,31 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Yang/summary.md</t>
+          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="K30" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="M30" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -2265,17 +2265,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sharma.sbml</t>
+          <t>Karrer.sbml</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sharma2018_BPA_Human</t>
+          <t>Karrer2018_BPA_Human</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>Karrer</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2290,53 +2290,53 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
+          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="M31" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="N31" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Karrer.sbml</t>
+          <t>ElMasri2008.sbml</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Karrer2018_BPA_Human</t>
+          <t>ElMasri2008_As_Human</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Karrer</t>
+          <t>ElMasri 2008</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2346,58 +2346,58 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="K32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L32" t="n">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="M32" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="N32" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="O32" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ElMasri2008.sbml</t>
+          <t>Ruiz2010_Male.sbml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ElMasri2008_As_Human</t>
+          <t>Ruiz2010_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ElMasri 2008</t>
+          <t>Ruiz 2010_Female</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2412,43 +2412,43 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J33" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="K33" t="n">
         <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>78</v>
+        <v>15</v>
       </c>
       <c r="M33" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="N33" t="n">
-        <v>107</v>
+        <v>10</v>
       </c>
       <c r="O33" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ruiz2010_Male.sbml</t>
+          <t>Ruiz2010_Female.sbml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2509,17 +2509,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ruiz2010_Female.sbml</t>
+          <t>Pouillot2022.sbml</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>Pouillot2022_Cd_Human</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Female</t>
+          <t>Pouillot 2022</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2555,32 +2555,32 @@
         <v>2</v>
       </c>
       <c r="L35" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M35" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N35" t="n">
+        <v>7</v>
+      </c>
+      <c r="O35" t="n">
         <v>10</v>
-      </c>
-      <c r="O35" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Pouillot2022.sbml</t>
+          <t>Bechaux2014_Male.sbml</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Pouillot2022_Cd_Human</t>
+          <t>Bechaux2014_Cd_Human_Female</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Pouillot 2022</t>
+          <t>Bechaux 2014_Female</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2607,22 +2607,22 @@
         <v>9</v>
       </c>
       <c r="I36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J36" t="n">
         <v>9</v>
       </c>
       <c r="K36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M36" t="n">
         <v>12</v>
       </c>
       <c r="N36" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O36" t="n">
         <v>10</v>
@@ -2631,7 +2631,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Bechaux2014_Male.sbml</t>
+          <t>Bechaux2014_Female.sbml</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2692,17 +2692,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Bechaux2014_Female.sbml</t>
+          <t>OFlaherty2000.sbml</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>OFlaherty2000_Pb_Human</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>OFlaherty 2000</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2717,53 +2717,53 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
         <v>3</v>
       </c>
-      <c r="J38" t="n">
-        <v>9</v>
-      </c>
       <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>21</v>
+      </c>
+      <c r="M38" t="n">
         <v>3</v>
       </c>
-      <c r="L38" t="n">
-        <v>15</v>
-      </c>
-      <c r="M38" t="n">
-        <v>12</v>
-      </c>
       <c r="N38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="O38" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OFlaherty2000.sbml</t>
+          <t>OFlaherty2001.sbml</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb_Human</t>
+          <t>OFlaherty2001_Cr_Human</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OFlaherty 2000</t>
+          <t>OFlaherty 2001</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2778,53 +2778,53 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="M39" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="N39" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="O39" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OFlaherty2001.sbml</t>
+          <t>Ou2018.sbml</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>OFlaherty2001_Cr_Human</t>
+          <t>Ou2018_Hg_Human</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>OFlaherty 2001</t>
+          <t>Ou 2018</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2839,53 +2839,53 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L40" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M40" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N40" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="O40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ou2018.sbml</t>
+          <t>KjellstromNordberg1978.sbml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ou2018_Hg_Human</t>
+          <t>KjellstromNordberg1978_Cd_Human</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ou 2018</t>
+          <t>KjellstromNordberg 1978</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2900,19 +2900,19 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J41" t="n">
         <v>9</v>
@@ -2921,32 +2921,32 @@
         <v>2</v>
       </c>
       <c r="L41" t="n">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="M41" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N41" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="O41" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978.sbml</t>
+          <t>Carrier2001.sbml</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978_Cd_Human</t>
+          <t>Carrier2001_Hg_Human</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>KjellstromNordberg 1978</t>
+          <t>Carrier 2001</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2961,53 +2961,53 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>GI;Liver;Blood</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="M42" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="N42" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O42" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Carrier2001.sbml</t>
+          <t>Tebby2022.sbml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg_Human</t>
+          <t>Tebby2022_Pb_Human</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Carrier 2001</t>
+          <t>Tebby 2022</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3022,12 +3022,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>GI;Liver;Blood</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -3043,32 +3043,32 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="M43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N43" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O43" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tebby2022.sbml</t>
+          <t>Clewell1999.sbml</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb_Human</t>
+          <t>Clewell_Hg_Human</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Tebby 2022</t>
+          <t>Clewell 1999</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3083,53 +3083,53 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="M44" t="n">
+        <v>14</v>
+      </c>
+      <c r="N44" t="n">
+        <v>20</v>
+      </c>
+      <c r="O44" t="n">
         <v>2</v>
-      </c>
-      <c r="N44" t="n">
-        <v>5</v>
-      </c>
-      <c r="O44" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Clewell1999.sbml</t>
+          <t>Tonnelier.sbml</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Clewell_Hg_Human</t>
+          <t>Tonnelier2012_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Clewell 1999</t>
+          <t>Tonnelier</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3139,58 +3139,58 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
+          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J45" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L45" t="n">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="M45" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N45" t="n">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="O45" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Tonnelier.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Tonnelier2012_Chlorpyrifos_Human</t>
+          <t>Chen_Fenitrothion_Human</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tonnelier</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3205,12 +3205,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
+          <t>./models/oral/Pesticides/Chen/summary.md</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
+          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -3220,38 +3220,38 @@
         <v>5</v>
       </c>
       <c r="J46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L46" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="M46" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="N46" t="n">
-        <v>58</v>
+        <v>88</v>
       </c>
       <c r="O46" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Chen_Fenitrothion_Human</t>
+          <t>Wei_Permethrin_Human</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3266,25 +3266,25 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Chen/summary.md</t>
+          <t>./models/oral/Pesticides/Wei/summary.md</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
+          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I47" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J47" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K47" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L47" t="n">
         <v>31</v>
@@ -3293,26 +3293,26 @@
         <v>31</v>
       </c>
       <c r="N47" t="n">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="O47" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Wei.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Wei_Permethrin_Human</t>
+          <t>Bouchard2010_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3327,53 +3327,53 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Wei/summary.md</t>
+          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
+          <t>Gut;Blood;Rest</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I48" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J48" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K48" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="L48" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="M48" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="N48" t="n">
-        <v>104</v>
+        <v>8</v>
       </c>
       <c r="O48" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Bouchard.sbml</t>
+          <t>Moreau_Deltamethrin.sbml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bouchard2010_Chlorpyrifos_Human</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Bouchard</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3388,43 +3388,43 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Gut;Blood;Rest</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I49" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J49" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K49" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L49" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="M49" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="N49" t="n">
-        <v>8</v>
+        <v>108</v>
       </c>
       <c r="O49" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin.sbml</t>
+          <t>Moreau_Carbaryl.sbml</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3485,17 +3485,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl.sbml</t>
+          <t>Mallick.sbml</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>Mallick2020_Pyrethroids_Human</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl</t>
+          <t>Mallick</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3510,53 +3510,53 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/Pesticides/Mallick/summary.md</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
         </is>
       </c>
       <c r="H51" t="n">
+        <v>6</v>
+      </c>
+      <c r="I51" t="n">
+        <v>6</v>
+      </c>
+      <c r="J51" t="n">
         <v>7</v>
       </c>
-      <c r="I51" t="n">
+      <c r="K51" t="n">
         <v>7</v>
       </c>
-      <c r="J51" t="n">
-        <v>9</v>
-      </c>
-      <c r="K51" t="n">
-        <v>9</v>
-      </c>
       <c r="L51" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M51" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N51" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="O51" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mallick.sbml</t>
+          <t>Zhao.sbml</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Mallick2020_Pyrethroids_Human</t>
+          <t>Zhao2019_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Mallick</t>
+          <t>Zhao</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3571,19 +3571,19 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Mallick/summary.md</t>
+          <t>./models/oral/Pesticides/Zhao/summary.md</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I52" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J52" t="n">
         <v>7</v>
@@ -3592,32 +3592,32 @@
         <v>7</v>
       </c>
       <c r="L52" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="M52" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="N52" t="n">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="O52" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Zhao.sbml</t>
+          <t>Zwartsen.sbml</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Zhao2019_Chlorpyrifos_Human</t>
+          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Zhao</t>
+          <t>Zwartsen</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3632,19 +3632,19 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zhao/summary.md</t>
+          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I53" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J53" t="n">
         <v>7</v>
@@ -3653,32 +3653,32 @@
         <v>7</v>
       </c>
       <c r="L53" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="M53" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="N53" t="n">
-        <v>52</v>
+        <v>114</v>
       </c>
       <c r="O53" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Zwartsen.sbml</t>
+          <t>Godin.sbml</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
+          <t>Godin_Pyrethroid_Human</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Zwartsen</t>
+          <t>Godin</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3693,53 +3693,53 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
+          <t>./models/oral/Pesticides/Godin/summary.md</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
+          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I54" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J54" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K54" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L54" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="M54" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="N54" t="n">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="O54" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Godin.sbml</t>
+          <t>Timchalk.sbml</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Godin_Pyrethroid_Human</t>
+          <t>Timchalk2002_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Godin</t>
+          <t>Timchalk</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3754,53 +3754,53 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Godin/summary.md</t>
+          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I55" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J55" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K55" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L55" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="M55" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="N55" t="n">
-        <v>106</v>
+        <v>46</v>
       </c>
       <c r="O55" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Timchalk.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Timchalk2002_Chlorpyrifos_Human</t>
+          <t>Chen2022_PFOS_Human</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Timchalk</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3810,58 +3810,58 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+          <t>./models/oral/PFAS/Chen/summary.md</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H56" t="n">
+        <v>6</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>6</v>
+      </c>
+      <c r="K56" t="n">
+        <v>2</v>
+      </c>
+      <c r="L56" t="n">
+        <v>29</v>
+      </c>
+      <c r="M56" t="n">
+        <v>7</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
         <v>3</v>
-      </c>
-      <c r="I56" t="n">
-        <v>3</v>
-      </c>
-      <c r="J56" t="n">
-        <v>5</v>
-      </c>
-      <c r="K56" t="n">
-        <v>5</v>
-      </c>
-      <c r="L56" t="n">
-        <v>23</v>
-      </c>
-      <c r="M56" t="n">
-        <v>23</v>
-      </c>
-      <c r="N56" t="n">
-        <v>46</v>
-      </c>
-      <c r="O56" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>ChouLin.sbml</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Chen2022_PFOS_Human</t>
+          <t>Chou_Lin2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>ChouLin</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Chen/summary.md</t>
+          <t>./models/oral/PFAS/ChouLin/summary.md</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3912,17 +3912,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ChouLin.sbml</t>
+          <t>Husoy.sbml</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Chou_Lin2021_PFOS_Human</t>
+          <t>Husoy2024_PFOA_Human</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ChouLin</t>
+          <t>Husoy</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3937,34 +3937,34 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+          <t>./models/oral/PFAS/Husoy/summary.md</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>GI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K58" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L58" t="n">
         <v>29</v>
       </c>
       <c r="M58" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O58" t="n">
         <v>3</v>
@@ -3973,17 +3973,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Husoy.sbml</t>
+          <t>Worley.sbml</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Husoy2024_PFOA_Human</t>
+          <t>Worley2017_PFOA_Human</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Husoy</t>
+          <t>Worley</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3998,34 +3998,34 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Husoy/summary.md</t>
+          <t>./models/oral/PFAS/Worley/summary.md</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L59" t="n">
         <v>29</v>
       </c>
       <c r="M59" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N59" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O59" t="n">
         <v>3</v>
@@ -4034,17 +4034,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Worley.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Worley2017_PFOA_Human</t>
+          <t>Deepika2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Worley</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4059,31 +4059,31 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Worley/summary.md</t>
+          <t>./models/oral/PFAS/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K60" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="M60" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="N60" t="n">
         <v>0</v>
@@ -4095,17 +4095,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Loccisano.sbml</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Deepika2021_PFOS_Human</t>
+          <t>Loccisano2011_PFAS_Human</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Loccisano</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Deepika/summary.md</t>
+          <t>./models/oral/PFAS/Loccisano/summary.md</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -4150,67 +4150,6 @@
         <v>0</v>
       </c>
       <c r="O61" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Loccisano.sbml</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Loccisano2011_PFAS_Human</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Loccisano</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>oral</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>PFAS</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>./models/oral/PFAS/Loccisano/summary.md</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>GI;Liver;Plasma;Rest</t>
-        </is>
-      </c>
-      <c r="H62" t="n">
-        <v>4</v>
-      </c>
-      <c r="I62" t="n">
-        <v>0</v>
-      </c>
-      <c r="J62" t="n">
-        <v>4</v>
-      </c>
-      <c r="K62" t="n">
-        <v>0</v>
-      </c>
-      <c r="L62" t="n">
-        <v>25</v>
-      </c>
-      <c r="M62" t="n">
-        <v>1</v>
-      </c>
-      <c r="N62" t="n">
-        <v>0</v>
-      </c>
-      <c r="O62" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 94663ad with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -1765,7 +1765,7 @@
         <v>28</v>
       </c>
       <c r="M22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N22" t="n">
         <v>0</v>
@@ -1826,7 +1826,7 @@
         <v>22</v>
       </c>
       <c r="M23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
         <v>0</v>
@@ -1875,19 +1875,19 @@
         <v>7</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
         <v>9</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
         <v>34</v>
       </c>
       <c r="M24" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="N24" t="n">
         <v>1</v>
@@ -2009,7 +2009,7 @@
         <v>36</v>
       </c>
       <c r="M26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
@@ -2131,7 +2131,7 @@
         <v>30</v>
       </c>
       <c r="M28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
@@ -2192,7 +2192,7 @@
         <v>59</v>
       </c>
       <c r="M29" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
@@ -2247,13 +2247,13 @@
         <v>8</v>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
         <v>37</v>
       </c>
       <c r="M30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -2314,7 +2314,7 @@
         <v>59</v>
       </c>
       <c r="M31" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed 6d3faeb with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1448,25 +1448,25 @@
         <v>12</v>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>16</v>
       </c>
       <c r="K17" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="M17" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18">
@@ -1509,25 +1509,25 @@
         <v>14</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
         <v>20</v>
       </c>
       <c r="K18" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>87</v>
       </c>
       <c r="M18" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19">
@@ -1570,25 +1570,25 @@
         <v>13</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
         <v>15</v>
       </c>
       <c r="K19" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M19" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -1637,19 +1637,19 @@
         <v>6</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
         <v>20</v>
       </c>
       <c r="M20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -1692,22 +1692,22 @@
         <v>8</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
         <v>9</v>
       </c>
       <c r="K21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M21" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="N21" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O21" t="n">
         <v>17</v>
@@ -2387,17 +2387,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ruiz2010_Male.sbml</t>
+          <t>Pouillot2022.sbml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>Pouillot2022_Cd_Human</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Female</t>
+          <t>Pouillot 2022</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2412,53 +2412,53 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>GI;Intestinal_Tissue;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake;Feces;Urine</t>
         </is>
       </c>
       <c r="H33" t="n">
         <v>9</v>
       </c>
       <c r="I33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
         <v>9</v>
       </c>
       <c r="K33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="M33" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N33" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O33" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ruiz2010_Female.sbml</t>
+          <t>OFlaherty2000.sbml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Ruiz2010_Cd_Human_Female</t>
+          <t>OFlaherty2000_Pb_Human</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ruiz 2010_Female</t>
+          <t>OFlaherty 2000</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2473,53 +2473,53 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ruiz2010/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="M34" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="N34" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O34" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Pouillot2022.sbml</t>
+          <t>OFlaherty2001.sbml</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pouillot2022_Cd_Human</t>
+          <t>OFlaherty2001_Cr_Human</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Pouillot 2022</t>
+          <t>OFlaherty 2001</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2534,53 +2534,53 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="M35" t="n">
         <v>12</v>
       </c>
       <c r="N35" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="O35" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Bechaux2014_Male.sbml</t>
+          <t>Ou2018.sbml</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>Ou2018_Hg_Human</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>Ou 2018</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2595,53 +2595,53 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
         <v>9</v>
       </c>
       <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>42</v>
+      </c>
+      <c r="M36" t="n">
         <v>3</v>
       </c>
-      <c r="L36" t="n">
-        <v>15</v>
-      </c>
-      <c r="M36" t="n">
-        <v>12</v>
-      </c>
       <c r="N36" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="O36" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Bechaux2014_Female.sbml</t>
+          <t>KjellstromNordberg1978.sbml</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Bechaux2014_Cd_Human_Female</t>
+          <t>KjellstromNordberg1978_Cd_Human</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bechaux 2014_Female</t>
+          <t>KjellstromNordberg 1978</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2656,34 +2656,34 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Bechaux2014/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>GI;Intestinal_Tissue;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake;Feces;Urine</t>
         </is>
       </c>
       <c r="H37" t="n">
         <v>9</v>
       </c>
       <c r="I37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
         <v>9</v>
       </c>
       <c r="K37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="M37" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N37" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="O37" t="n">
         <v>10</v>
@@ -2692,17 +2692,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OFlaherty2000.sbml</t>
+          <t>Carrier2001.sbml</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb_Human</t>
+          <t>Carrier2001_Hg_Human</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>OFlaherty 2000</t>
+          <t>Carrier 2001</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2717,53 +2717,53 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GI;Blood;Rest;Hair;Liver</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="M38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OFlaherty2001.sbml</t>
+          <t>Tebby2022.sbml</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>OFlaherty2001_Cr_Human</t>
+          <t>Tebby2022_Pb_Human</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OFlaherty 2001</t>
+          <t>Tebby 2022</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2778,53 +2778,53 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H39" t="n">
+        <v>3</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>3</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>21</v>
+      </c>
+      <c r="M39" t="n">
+        <v>2</v>
+      </c>
+      <c r="N39" t="n">
+        <v>5</v>
+      </c>
+      <c r="O39" t="n">
         <v>6</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="n">
-        <v>12</v>
-      </c>
-      <c r="K39" t="n">
-        <v>0</v>
-      </c>
-      <c r="L39" t="n">
-        <v>30</v>
-      </c>
-      <c r="M39" t="n">
-        <v>12</v>
-      </c>
-      <c r="N39" t="n">
-        <v>19</v>
-      </c>
-      <c r="O39" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ou2018.sbml</t>
+          <t>Clewell1999.sbml</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ou2018_Hg_Human</t>
+          <t>Clewell_Hg_Human</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ou 2018</t>
+          <t>Clewell 1999</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Ou2018/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2857,7 +2857,7 @@
         <v>9</v>
       </c>
       <c r="K40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L40" t="n">
         <v>42</v>
@@ -2866,26 +2866,26 @@
         <v>14</v>
       </c>
       <c r="N40" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978.sbml</t>
+          <t>Tonnelier.sbml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978_Cd_Human</t>
+          <t>Tonnelier2012_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>KjellstromNordberg 1978</t>
+          <t>Tonnelier</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2895,58 +2895,58 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
+          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Liver;Kidney;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake</t>
+          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I41" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J41" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L41" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M41" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="N41" t="n">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="O41" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Carrier2001.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg_Human</t>
+          <t>Chen_Fenitrothion_Human</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Carrier 2001</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2956,58 +2956,58 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
+          <t>./models/oral/Pesticides/Chen/summary.md</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>GI;Liver;Blood</t>
+          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J42" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L42" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="M42" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="N42" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="O42" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tebby2022.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb_Human</t>
+          <t>Wei_Permethrin_Human</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Tebby 2022</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3017,58 +3017,58 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
+          <t>./models/oral/Pesticides/Wei/summary.md</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J43" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L43" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="M43" t="n">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="N43" t="n">
-        <v>5</v>
+        <v>104</v>
       </c>
       <c r="O43" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Clewell1999.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Clewell_Hg_Human</t>
+          <t>Bouchard2010_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Clewell 1999</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3078,58 +3078,58 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
+          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>Gut;Blood;Rest</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K44" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L44" t="n">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="M44" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="N44" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="O44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tonnelier.sbml</t>
+          <t>Moerenhout.sbml</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Tonnelier2012_Chlorpyrifos_Human</t>
+          <t>Moerenhout2022_Pesticides_Human</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tonnelier</t>
+          <t>Moerenhout</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3144,53 +3144,53 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
+          <t>./models/oral/Pesticides/Moerenhout/summary.md</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Blood;Liver;Kidney;Rest;Urine;Feces</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="I45" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="K45" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="M45" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="N45" t="n">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="O45" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Moreau_Deltamethrin.sbml</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Chen_Fenitrothion_Human</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3205,53 +3205,53 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Chen/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I46" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J46" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K46" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L46" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="M46" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="N46" t="n">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="O46" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Wei.sbml</t>
+          <t>Moreau_Carbaryl.sbml</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Wei_Permethrin_Human</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3266,53 +3266,53 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Wei/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H47" t="n">
+        <v>7</v>
+      </c>
+      <c r="I47" t="n">
+        <v>7</v>
+      </c>
+      <c r="J47" t="n">
         <v>9</v>
       </c>
-      <c r="I47" t="n">
+      <c r="K47" t="n">
         <v>9</v>
       </c>
-      <c r="J47" t="n">
-        <v>11</v>
-      </c>
-      <c r="K47" t="n">
-        <v>11</v>
-      </c>
       <c r="L47" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="M47" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="N47" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="O47" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Bouchard.sbml</t>
+          <t>Mallick.sbml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Bouchard2010_Chlorpyrifos_Human</t>
+          <t>Mallick2020_Pyrethroids_Human</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Bouchard</t>
+          <t>Mallick</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3327,53 +3327,53 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
+          <t>./models/oral/Pesticides/Mallick/summary.md</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Gut;Blood;Rest</t>
+          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I48" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J48" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K48" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L48" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="M48" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="N48" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="O48" t="n">
-        <v>4</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin.sbml</t>
+          <t>Zhao.sbml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>Zhao2019_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl</t>
+          <t>Zhao</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3388,53 +3388,53 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/Pesticides/Zhao/summary.md</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H49" t="n">
+        <v>4</v>
+      </c>
+      <c r="I49" t="n">
+        <v>4</v>
+      </c>
+      <c r="J49" t="n">
         <v>7</v>
       </c>
-      <c r="I49" t="n">
+      <c r="K49" t="n">
         <v>7</v>
       </c>
-      <c r="J49" t="n">
-        <v>9</v>
-      </c>
-      <c r="K49" t="n">
-        <v>9</v>
-      </c>
       <c r="L49" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="M49" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="N49" t="n">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="O49" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl.sbml</t>
+          <t>Zwartsen.sbml</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl</t>
+          <t>Zwartsen</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3449,53 +3449,53 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H50" t="n">
+        <v>5</v>
+      </c>
+      <c r="I50" t="n">
+        <v>5</v>
+      </c>
+      <c r="J50" t="n">
         <v>7</v>
       </c>
-      <c r="I50" t="n">
+      <c r="K50" t="n">
         <v>7</v>
       </c>
-      <c r="J50" t="n">
-        <v>9</v>
-      </c>
-      <c r="K50" t="n">
-        <v>9</v>
-      </c>
       <c r="L50" t="n">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="M50" t="n">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="N50" t="n">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="O50" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Mallick.sbml</t>
+          <t>Godin.sbml</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Mallick2020_Pyrethroids_Human</t>
+          <t>Godin_Pyrethroid_Human</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Mallick</t>
+          <t>Godin</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3510,53 +3510,53 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Mallick/summary.md</t>
+          <t>./models/oral/Pesticides/Godin/summary.md</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
+          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I51" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J51" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K51" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L51" t="n">
+        <v>34</v>
+      </c>
+      <c r="M51" t="n">
+        <v>34</v>
+      </c>
+      <c r="N51" t="n">
+        <v>106</v>
+      </c>
+      <c r="O51" t="n">
         <v>36</v>
-      </c>
-      <c r="M51" t="n">
-        <v>36</v>
-      </c>
-      <c r="N51" t="n">
-        <v>100</v>
-      </c>
-      <c r="O51" t="n">
-        <v>35</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Zhao.sbml</t>
+          <t>Timchalk.sbml</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Zhao2019_Chlorpyrifos_Human</t>
+          <t>Timchalk2002_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Zhao</t>
+          <t>Timchalk</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3571,34 +3571,34 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zhao/summary.md</t>
+          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J52" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K52" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L52" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="M52" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="N52" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="O52" t="n">
         <v>17</v>
@@ -3607,17 +3607,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Zwartsen.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
+          <t>Chen2022_PFOS_Human</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Zwartsen</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3627,58 +3627,58 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
+          <t>./models/oral/PFAS/Chen/summary.md</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I53" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
+        <v>6</v>
+      </c>
+      <c r="K53" t="n">
+        <v>2</v>
+      </c>
+      <c r="L53" t="n">
+        <v>29</v>
+      </c>
+      <c r="M53" t="n">
         <v>7</v>
       </c>
-      <c r="K53" t="n">
-        <v>7</v>
-      </c>
-      <c r="L53" t="n">
-        <v>57</v>
-      </c>
-      <c r="M53" t="n">
-        <v>57</v>
-      </c>
       <c r="N53" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="O53" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Godin.sbml</t>
+          <t>ChouLin.sbml</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Godin_Pyrethroid_Human</t>
+          <t>Chou_Lin2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Godin</t>
+          <t>ChouLin</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3688,58 +3688,58 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Godin/summary.md</t>
+          <t>./models/oral/PFAS/ChouLin/summary.md</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I54" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K54" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L54" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="M54" t="n">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="N54" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="O54" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Timchalk.sbml</t>
+          <t>Husoy.sbml</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Timchalk2002_Chlorpyrifos_Human</t>
+          <t>Husoy2024_PFOA_Human</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Timchalk</t>
+          <t>Husoy</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3749,58 +3749,58 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+          <t>./models/oral/PFAS/Husoy/summary.md</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H55" t="n">
+        <v>5</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>5</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="n">
+        <v>29</v>
+      </c>
+      <c r="M55" t="n">
         <v>3</v>
       </c>
-      <c r="I55" t="n">
+      <c r="N55" t="n">
+        <v>2</v>
+      </c>
+      <c r="O55" t="n">
         <v>3</v>
-      </c>
-      <c r="J55" t="n">
-        <v>5</v>
-      </c>
-      <c r="K55" t="n">
-        <v>5</v>
-      </c>
-      <c r="L55" t="n">
-        <v>23</v>
-      </c>
-      <c r="M55" t="n">
-        <v>23</v>
-      </c>
-      <c r="N55" t="n">
-        <v>46</v>
-      </c>
-      <c r="O55" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Worley.sbml</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Chen2022_PFOS_Human</t>
+          <t>Worley2017_PFOA_Human</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Worley</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Chen/summary.md</t>
+          <t>./models/oral/PFAS/Worley/summary.md</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3851,17 +3851,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ChouLin.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Chou_Lin2021_PFOS_Human</t>
+          <t>Deepika2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ChouLin</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3876,31 +3876,31 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+          <t>./models/oral/PFAS/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K57" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L57" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="M57" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="N57" t="n">
         <v>0</v>
@@ -3912,17 +3912,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Husoy.sbml</t>
+          <t>Loccisano.sbml</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Husoy2024_PFOA_Human</t>
+          <t>Loccisano2011_PFAS_Human</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Husoy</t>
+          <t>Loccisano</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3937,219 +3937,36 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Husoy/summary.md</t>
+          <t>./models/oral/PFAS/Loccisano/summary.md</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest;Feces</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
       </c>
       <c r="L58" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="M58" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O58" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Worley.sbml</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Worley2017_PFOA_Human</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Worley</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>oral</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>PFAS</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>./models/oral/PFAS/Worley/summary.md</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
-        </is>
-      </c>
-      <c r="H59" t="n">
-        <v>6</v>
-      </c>
-      <c r="I59" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" t="n">
-        <v>6</v>
-      </c>
-      <c r="K59" t="n">
-        <v>2</v>
-      </c>
-      <c r="L59" t="n">
-        <v>29</v>
-      </c>
-      <c r="M59" t="n">
-        <v>7</v>
-      </c>
-      <c r="N59" t="n">
-        <v>0</v>
-      </c>
-      <c r="O59" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Deepika.sbml</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Deepika2021_PFOS_Human</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Deepika</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>oral</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>PFAS</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>./models/oral/PFAS/Deepika/summary.md</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>GI;Liver;Plasma;Rest</t>
-        </is>
-      </c>
-      <c r="H60" t="n">
-        <v>4</v>
-      </c>
-      <c r="I60" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" t="n">
-        <v>4</v>
-      </c>
-      <c r="K60" t="n">
-        <v>0</v>
-      </c>
-      <c r="L60" t="n">
-        <v>25</v>
-      </c>
-      <c r="M60" t="n">
-        <v>1</v>
-      </c>
-      <c r="N60" t="n">
-        <v>0</v>
-      </c>
-      <c r="O60" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Loccisano.sbml</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Loccisano2011_PFAS_Human</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Loccisano</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>oral</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>PFAS</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>./models/oral/PFAS/Loccisano/summary.md</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>GI;Liver;Plasma;Rest</t>
-        </is>
-      </c>
-      <c r="H61" t="n">
-        <v>4</v>
-      </c>
-      <c r="I61" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" t="n">
-        <v>4</v>
-      </c>
-      <c r="K61" t="n">
-        <v>0</v>
-      </c>
-      <c r="L61" t="n">
-        <v>25</v>
-      </c>
-      <c r="M61" t="n">
-        <v>1</v>
-      </c>
-      <c r="N61" t="n">
-        <v>0</v>
-      </c>
-      <c r="O61" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 758eeca with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -3650,13 +3650,13 @@
         <v>6</v>
       </c>
       <c r="K53" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L53" t="n">
         <v>29</v>
       </c>
       <c r="M53" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N53" t="n">
         <v>0</v>
@@ -3711,13 +3711,13 @@
         <v>6</v>
       </c>
       <c r="K54" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L54" t="n">
         <v>29</v>
       </c>
       <c r="M54" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N54" t="n">
         <v>0</v>
@@ -3778,7 +3778,7 @@
         <v>29</v>
       </c>
       <c r="M55" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N55" t="n">
         <v>2</v>
@@ -3833,13 +3833,13 @@
         <v>6</v>
       </c>
       <c r="K56" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L56" t="n">
         <v>29</v>
       </c>
       <c r="M56" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N56" t="n">
         <v>0</v>
@@ -3900,7 +3900,7 @@
         <v>25</v>
       </c>
       <c r="M57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N57" t="n">
         <v>0</v>
@@ -3961,7 +3961,7 @@
         <v>25</v>
       </c>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N58" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed c0b675a with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -496,200 +496,200 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>model_C_inh_exh_art_ven.sbml</t>
+          <t>dermal-steady-state-Dancik-based.sbml</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>inhalation_C_art_ven</t>
+          <t>Dermal_Diffusion_Dancik2013</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>model_C_inh_exh_art_ven</t>
+          <t>dermal-steady-state-Dancik-based</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>inhalation</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_C_alveolar_lung/summary.md</t>
+          <t>./models/dermal/Other/dermal-steady-state-Dancik-based/summary.md</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung;Bloodlung</t>
+          <t>Stratum_Corneum;Viable_Epidermis;Dermis</t>
         </is>
       </c>
       <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N2" t="n">
+        <v>34</v>
+      </c>
+      <c r="O2" t="n">
         <v>6</v>
-      </c>
-      <c r="I2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K2" t="n">
-        <v>5</v>
-      </c>
-      <c r="L2" t="n">
-        <v>22</v>
-      </c>
-      <c r="M2" t="n">
-        <v>21</v>
-      </c>
-      <c r="N2" t="n">
-        <v>22</v>
-      </c>
-      <c r="O2" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven.sbml</t>
+          <t>dermal-simple-Tonnelier-based.sbml</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>inhalation_B_art_ven</t>
+          <t>Dermal_PBK_Tonnelier_Simplified</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>model_B_inh_exh_art_ven</t>
+          <t>dermal-simple-Tonnelier-based</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>inhalation</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
+          <t>./models/dermal/Pesticides/Tonnelier/summary.md</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody;Lung</t>
+          <t>DermalAbsorptionCompartment;PortalVeinBlood;Liver;SystemicCompartment;RenalExcretion</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>5</v>
       </c>
       <c r="I3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
         <v>5</v>
       </c>
       <c r="K3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="M3" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="N3" t="n">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="O3" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>model_A_inh_exh_art_ven.sbml</t>
+          <t>Dermal_APM_CarrierBrunet1999_DermalOnly.sbml</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>inhalation_A_art_ven</t>
+          <t>Dermal_APM_CarrierBrunet1999_DermalOnly</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>model_A_inh_exh_art_ven</t>
+          <t>Dermal_APM_CarrierBrunet 1999_DermalOnly</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>inhalation</t>
+          <t>dermal</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
+          <t>./models/dermal/Pesticides/Carrier_Brunet/summary.md</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Air;Arterial;Venous;RestofBody</t>
+          <t>Skin;RestBody;Urine;NonObservedExcr</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" t="n">
         <v>4</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="M4" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="N4" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="O4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BPA_Dermal_simple-Hu-based.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BPA_Dermal_PBK_Hu_layered</t>
+          <t>Bouchard2005_DermalOnly_Simplified</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BPA_Dermal_simple-Hu-based</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -699,58 +699,58 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>./models/dermal/Bisphenols/Hu/summary.md</t>
+          <t>./models/dermal/Pesticides/Bouchard/summary.md</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SurfaceDepot;ExposedVE;Follicle;UnexposedSkin;Plasma;Restbody;Urine</t>
+          <t>SkinSurf;Blood;RestOfBody;Urine</t>
         </is>
       </c>
       <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L5" t="n">
         <v>7</v>
       </c>
-      <c r="I5" t="n">
-        <v>2</v>
-      </c>
-      <c r="J5" t="n">
+      <c r="M5" t="n">
         <v>7</v>
       </c>
-      <c r="K5" t="n">
-        <v>2</v>
-      </c>
-      <c r="L5" t="n">
-        <v>62</v>
-      </c>
-      <c r="M5" t="n">
-        <v>26</v>
-      </c>
       <c r="N5" t="n">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="O5" t="n">
-        <v>37</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>dermal-simple-model-Karrer-based.sbml</t>
+          <t>dermal-simple-Timchalk-based.sbml</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BPA_Dermal_Simplified_Karrer</t>
+          <t>Dermal_CPF_Timchalk2002_Simplified</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>dermal-simple-model-Karrer-based</t>
+          <t>dermal-simple-Timchalk-based</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -760,58 +760,58 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>./models/dermal/Bisphenols/Karrer/summary.md</t>
+          <t>./models/dermal/Pesticides/Timchalk/summary.md</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>SurfaceDepot;Skin;Plasma;Restbody;Urine</t>
+          <t>Skin;ArterialBlood;VenousBlood;RestOfBody;Elimination</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="M6" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="N6" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="O6" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dermal-simple-Tonnelier-based.sbml</t>
+          <t>Poet.sbml</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dermal_PBK_Tonnelier_Simplified</t>
+          <t>Poet2014_DermalOnly_SimplifiedCPF</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>dermal-simple-Tonnelier-based</t>
+          <t>Poet</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -826,12 +826,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>./models/dermal/Pesticides/Tonnelier/summary.md</t>
+          <t>./models/dermal/Pesticides/Poet/summary.md</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>DermalAbsorptionCompartment;PortalVeinBlood;Liver;SystemicCompartment;RenalExcretion</t>
+          <t>Skin;ArterialBlood;VenousBlood;RestOfBody;Elimination</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -841,38 +841,38 @@
         <v>5</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L7" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="M7" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="N7" t="n">
-        <v>53</v>
+        <v>100</v>
       </c>
       <c r="O7" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wei.sbml</t>
+          <t>dermal-simple-Tornero-Velez-based.sbml</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dermal_PBK_Wei_Simplified</t>
+          <t>permethrin_dermal_minPBK</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>dermal-simple-Tornero-Velez-based</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -887,53 +887,53 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>./models/dermal/Pesticides/Wei/summary.md</t>
+          <t>./models/dermal/Pesticides/Tornero-Velez/summary.md</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>default_compartment;Skin;Blood;RestOfBody;UrinaryExcretion</t>
+          <t>SkinSurface;StratumCorneum;ViableEpidermis;ArterialBlood;VenousBlood;UrinaryExcretion;RestOfBody</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L8" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="M8" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="N8" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="O8" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bouchard.sbml</t>
+          <t>dermal-simple-Quindroit-based.sbml</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bouchard2005_DermalOnly_Simplified</t>
+          <t>Dermal_PBK_Quindroit_Simplified</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bouchard</t>
+          <t>dermal-simple-Quindroit-based</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -948,53 +948,53 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>./models/dermal/Pesticides/Bouchard/summary.md</t>
+          <t>./models/dermal/Pesticides/Quindroit/summary.md</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SkinSurf;Blood;RestOfBody;Urine</t>
+          <t>SkinSurface;StratumCorneum;Skin;ArterialBlood;VenousBlood;UrinaryTrack;RestOfBody</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L9" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="M9" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="N9" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="O9" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dermal-simple-Quindroit-based.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dermal_PBK_Quindroit_Simplified</t>
+          <t>Dermal_PBK_Wei_Simplified</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>dermal-simple-Quindroit-based</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1009,53 +1009,53 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>./models/dermal/Pesticides/Quindroit/summary.md</t>
+          <t>./models/dermal/Pesticides/Wei/summary.md</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SkinSurface;StratumCorneum;Skin;ArterialBlood;VenousBlood;UrinaryTrack;RestOfBody</t>
+          <t>default_compartment;Skin;Blood;RestOfBody;UrinaryExcretion</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="M10" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="N10" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="O10" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dermal_APM_CarrierBrunet1999_DermalOnly.sbml</t>
+          <t>PFOA_dermal-simple-model-Husoy-based.sbml</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dermal_APM_CarrierBrunet1999_DermalOnly</t>
+          <t>Husoy2023_Dermal</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dermal_APM_CarrierBrunet 1999_DermalOnly</t>
+          <t>PFOA_dermal-simple-model-Husoy-based</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1065,58 +1065,58 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>./models/dermal/Pesticides/Carrier_Brunet/summary.md</t>
+          <t>./models/dermal/PFAS/Husoy/summary.md</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Skin;RestBody;Urine;NonObservedExcr</t>
+          <t>Skin;Plasma;RestBody;Kidney;Urine</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="M11" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="N11" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="O11" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dermal-simple-Tornero-Velez-based.sbml</t>
+          <t>BPA_Dermal_simple-Hu-based.sbml</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>permethrin_dermal_minPBK</t>
+          <t>BPA_Dermal_PBK_Hu_layered</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>dermal-simple-Tornero-Velez-based</t>
+          <t>BPA_Dermal_simple-Hu-based</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1126,58 +1126,58 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>./models/dermal/Pesticides/Tornero-Velez/summary.md</t>
+          <t>./models/dermal/Bisphenols/Hu/summary.md</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SkinSurface;StratumCorneum;ViableEpidermis;ArterialBlood;VenousBlood;UrinaryExcretion;RestOfBody</t>
+          <t>SurfaceDepot;ExposedVE;Follicle;UnexposedSkin;Plasma;Restbody;Urine</t>
         </is>
       </c>
       <c r="H12" t="n">
         <v>7</v>
       </c>
       <c r="I12" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>7</v>
       </c>
       <c r="K12" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L12" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="M12" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="N12" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="O12" t="n">
-        <v>13</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Poet.sbml</t>
+          <t>dermal-simple-model-Karrer-based.sbml</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Poet2014_DermalOnly_SimplifiedCPF</t>
+          <t>BPA_Dermal_Simplified_Karrer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Poet</t>
+          <t>dermal-simple-model-Karrer-based</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1187,17 +1187,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>./models/dermal/Pesticides/Poet/summary.md</t>
+          <t>./models/dermal/Bisphenols/Karrer/summary.md</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Skin;ArterialBlood;VenousBlood;RestOfBody;Elimination</t>
+          <t>SurfaceDepot;Skin;Plasma;Restbody;Urine</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -1207,221 +1207,221 @@
         <v>5</v>
       </c>
       <c r="J13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L13" t="n">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="M13" t="n">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="N13" t="n">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="O13" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dermal-simple-Timchalk-based.sbml</t>
+          <t>model_C_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dermal_CPF_Timchalk2002_Simplified</t>
+          <t>Inhalation_C_art_ven</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>dermal-simple-Timchalk-based</t>
+          <t>model_C_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>dermal</t>
+          <t>inhalation</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>./models/dermal/Pesticides/Timchalk/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_C_alveolar_lung/summary.md</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Skin;ArterialBlood;VenousBlood;RestOfBody;Elimination</t>
+          <t>Air;Arterial;Venous;RestofBody;Pulmonary1;Pulmonary2;Metabolite</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>7</v>
       </c>
       <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>30</v>
+      </c>
+      <c r="M14" t="n">
         <v>3</v>
       </c>
-      <c r="L14" t="n">
-        <v>27</v>
-      </c>
-      <c r="M14" t="n">
-        <v>20</v>
-      </c>
       <c r="N14" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="O14" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PFOA_dermal-simple-model-Husoy-based.sbml</t>
+          <t>model_B_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Husoy2023_Dermal</t>
+          <t>Inhalation_B_art_ven</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PFOA_dermal-simple-model-Husoy-based</t>
+          <t>model_B_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>dermal</t>
+          <t>inhalation</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>./models/dermal/PFAS/Husoy/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_B_lung/summary.md</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Skin;Plasma;RestBody;Kidney;Urine</t>
+          <t>Air;Arterial;Venous;RestofBody;Pulmonary;Metabolite</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="M15" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="N15" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="O15" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dermal-steady-state-Dancik-based.sbml</t>
+          <t>model_A_inh_exh_art_ven.sbml</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dermal_Diffusion_Dancik2013</t>
+          <t>Inhalation_A_art_ven</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>dermal-steady-state-Dancik-based</t>
+          <t>model_A_inh_exh_art_ven</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>dermal</t>
+          <t>inhalation</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>./models/dermal/Other/dermal-steady-state-Dancik-based/summary.md</t>
+          <t>./models/inhalation/Generic/Structure_A_direct_blood/summary.md</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Stratum_Corneum;Viable_Epidermis;Dermis</t>
+          <t>Air;Arterial;Venous;RestofBody</t>
         </is>
       </c>
       <c r="H16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>16</v>
+      </c>
+      <c r="M16" t="n">
         <v>3</v>
       </c>
-      <c r="I16" t="n">
-        <v>3</v>
-      </c>
-      <c r="J16" t="n">
-        <v>3</v>
-      </c>
-      <c r="K16" t="n">
-        <v>3</v>
-      </c>
-      <c r="L16" t="n">
-        <v>10</v>
-      </c>
-      <c r="M16" t="n">
-        <v>10</v>
-      </c>
       <c r="N16" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="O16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mukherjee.sbml</t>
+          <t>Mallick.sbml</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mukherjee2014_Human_PBK</t>
+          <t>Mallick2020_Pyrethroids_Human</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mukherjee</t>
+          <t>Mallick</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1431,58 +1431,58 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
+          <t>./models/oral/Pesticides/Mallick/summary.md</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
+          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J17" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L17" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O17" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mendez_Catala.sbml</t>
+          <t>Zwartsen.sbml</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mandez_Catal_2021_Human_PBK</t>
+          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mendez_Catala</t>
+          <t>Zwartsen</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1492,58 +1492,58 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
+          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
+          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J18" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L18" t="n">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="O18" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval.sbml</t>
+          <t>Tonnelier.sbml</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GilbertSandoval</t>
+          <t>Tonnelier2012_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Gilbert_Sandoval</t>
+          <t>Tonnelier</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1553,58 +1553,58 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
+          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
+          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J19" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L19" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="O19" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Notenboom.sbml</t>
+          <t>Zhao.sbml</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Notenboom2023_DON_Human</t>
+          <t>Zhao2019_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Notenboom</t>
+          <t>Zhao</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1614,58 +1614,58 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
+          <t>./models/oral/Pesticides/Zhao/summary.md</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Lumen;Liver;Blood;Rest</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H20" t="n">
         <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L20" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="O20" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Wang.sbml</t>
+          <t>Moerenhout.sbml</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Wang2023_DON_Human</t>
+          <t>Moerenhout2022_Pesticides_Human</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wang</t>
+          <t>Moerenhout</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1675,58 +1675,58 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mycotoxins</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
+          <t>./models/oral/Pesticides/Moerenhout/summary.md</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Blood;Liver;Kidney;Rest;Urine;Feces</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>46</v>
+        <v>82</v>
       </c>
       <c r="M21" t="n">
         <v>3</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="O21" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shin.sbml</t>
+          <t>Bouchard.sbml</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Shin2004_BPA_Human</t>
+          <t>Bouchard2010_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Shin</t>
+          <t>Bouchard</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1736,58 +1736,58 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Shin/summary.md</t>
+          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
+          <t>Gut;Blood;Rest</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J22" t="n">
+        <v>4</v>
+      </c>
+      <c r="K22" t="n">
+        <v>4</v>
+      </c>
+      <c r="L22" t="n">
+        <v>4</v>
+      </c>
+      <c r="M22" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" t="n">
         <v>8</v>
       </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
-        <v>28</v>
-      </c>
-      <c r="M22" t="n">
-        <v>1</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0</v>
-      </c>
       <c r="O22" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mielke.sbml</t>
+          <t>Timchalk.sbml</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mielke2009_BPA_Human</t>
+          <t>Timchalk2002_Chlorpyrifos_Human</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mielke</t>
+          <t>Timchalk</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1797,58 +1797,58 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
+          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L23" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="O23" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Moreau.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Moreau2025_BPA_Human</t>
+          <t>Chen_Fenitrothion_Human</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Moreau</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1858,58 +1858,58 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
+          <t>./models/oral/Pesticides/Chen/summary.md</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H24" t="n">
+        <v>5</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" t="n">
         <v>7</v>
       </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>9</v>
-      </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L24" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="M24" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="N24" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="O24" t="n">
-        <v>5</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Deepika.sbml</t>
+          <t>Godin.sbml</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Deepika2022_BPA_Human</t>
+          <t>Godin_Pyrethroid_Human</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Deepika</t>
+          <t>Godin</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1919,58 +1919,58 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
+          <t>./models/oral/Pesticides/Godin/summary.md</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J25" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L25" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="O25" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Loizou.sbml</t>
+          <t>Moreau_Deltamethrin.sbml</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Loizou2022_BPA_Human</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Loizou</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1980,58 +1980,58 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J26" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L26" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="O26" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Christensen.sbml</t>
+          <t>Moreau_Carbaryl.sbml</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Christensen2013_BPA_Human</t>
+          <t>Moreau_Carbaryl_Human</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Christensen</t>
+          <t>Moreau_Carbaryl</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2041,58 +2041,58 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
+          <t>./models/oral/Pesticides/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Stomach;Blood;Bladder</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L27" t="n">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="O27" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Teeguarden.sbml</t>
+          <t>Wei.sbml</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Teeguarden2005_BPA_Human</t>
+          <t>Wei_Permethrin_Human</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Teeguarden</t>
+          <t>Wei</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2102,58 +2102,58 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>Pesticides</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
+          <t>./models/oral/Pesticides/Wei/summary.md</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>GILumen;Liver;Blood;Rest;Feces</t>
+          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J28" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L28" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="O28" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Yang.sbml</t>
+          <t>Worley.sbml</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yang2015_BPA_Human</t>
+          <t>Worley2017_PFOA_Human</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Yang</t>
+          <t>Worley</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2163,58 +2163,58 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Yang/summary.md</t>
+          <t>./models/oral/PFAS/Worley/summary.md</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>29</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
         <v>3</v>
-      </c>
-      <c r="L29" t="n">
-        <v>59</v>
-      </c>
-      <c r="M29" t="n">
-        <v>4</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sharma.sbml</t>
+          <t>Husoy.sbml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sharma2018_BPA_Human</t>
+          <t>Husoy2024_PFOA_Human</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sharma</t>
+          <t>Husoy</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2224,17 +2224,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
+          <t>./models/oral/PFAS/Husoy/summary.md</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Stomach;Liver;Plasma;Gut;Rest</t>
+          <t>GI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -2244,38 +2244,38 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O30" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Karrer.sbml</t>
+          <t>Chen.sbml</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Karrer2018_BPA_Human</t>
+          <t>Chen2022_PFOS_Human</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Karrer</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2285,58 +2285,58 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Bisphenols</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
+          <t>./models/oral/PFAS/Chen/summary.md</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="M31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ElMasri2008.sbml</t>
+          <t>ChouLin.sbml</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ElMasri2008_As_Human</t>
+          <t>Chou_Lin2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ElMasri 2008</t>
+          <t>ChouLin</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2346,58 +2346,58 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
+          <t>./models/oral/PFAS/ChouLin/summary.md</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="M32" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pouillot2022.sbml</t>
+          <t>Deepika.sbml</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pouillot2022_Cd_Human</t>
+          <t>Deepika2021_PFOS_Human</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Pouillot 2022</t>
+          <t>Deepika</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2407,58 +2407,58 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
+          <t>./models/oral/PFAS/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake;Feces;Urine</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="M33" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OFlaherty2000.sbml</t>
+          <t>Loccisano.sbml</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>OFlaherty2000_Pb_Human</t>
+          <t>Loccisano2011_PFAS_Human</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>OFlaherty 2000</t>
+          <t>Loccisano</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2468,58 +2468,58 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>PFAS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
+          <t>./models/oral/PFAS/Loccisano/summary.md</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>GI;Liver;Plasma;Rest</t>
         </is>
       </c>
       <c r="H34" t="n">
+        <v>4</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>4</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>25</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="n">
         <v>3</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>3</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" t="n">
-        <v>21</v>
-      </c>
-      <c r="M34" t="n">
-        <v>3</v>
-      </c>
-      <c r="N34" t="n">
-        <v>3</v>
-      </c>
-      <c r="O34" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OFlaherty2001.sbml</t>
+          <t>OFlaherty2000.sbml</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>OFlaherty2001_Cr_Human</t>
+          <t>OFlaherty2000_Pb_Human</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>OFlaherty 2001</t>
+          <t>OFlaherty 2000</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2534,37 +2534,37 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2000/summary.md</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H35" t="n">
+        <v>3</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>3</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>21</v>
+      </c>
+      <c r="M35" t="n">
+        <v>3</v>
+      </c>
+      <c r="N35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O35" t="n">
         <v>6</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>12</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="n">
-        <v>30</v>
-      </c>
-      <c r="M35" t="n">
-        <v>12</v>
-      </c>
-      <c r="N35" t="n">
-        <v>19</v>
-      </c>
-      <c r="O35" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -2631,17 +2631,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978.sbml</t>
+          <t>OFlaherty2001.sbml</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KjellstromNordberg1978_Cd_Human</t>
+          <t>OFlaherty2001_Cr_Human</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KjellstromNordberg 1978</t>
+          <t>OFlaherty 2001</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2656,53 +2656,53 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/OFlaherty2001/summary.md</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>GI;Intestinal_Tissue;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake;Feces;Urine</t>
+          <t>GI;Liver;Plasma;RBC;Rest;Feces</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
       </c>
       <c r="L37" t="n">
+        <v>30</v>
+      </c>
+      <c r="M37" t="n">
         <v>12</v>
       </c>
-      <c r="M37" t="n">
-        <v>11</v>
-      </c>
       <c r="N37" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="O37" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Carrier2001.sbml</t>
+          <t>Tebby2022.sbml</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Carrier2001_Hg_Human</t>
+          <t>Tebby2022_Pb_Human</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Carrier 2001</t>
+          <t>Tebby 2022</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2717,53 +2717,53 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>GI;Blood;Rest;Hair;Liver</t>
+          <t>Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H38" t="n">
+        <v>3</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>21</v>
+      </c>
+      <c r="M38" t="n">
+        <v>2</v>
+      </c>
+      <c r="N38" t="n">
         <v>5</v>
       </c>
-      <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="n">
-        <v>5</v>
-      </c>
-      <c r="K38" t="n">
-        <v>1</v>
-      </c>
-      <c r="L38" t="n">
-        <v>7</v>
-      </c>
-      <c r="M38" t="n">
-        <v>4</v>
-      </c>
-      <c r="N38" t="n">
-        <v>0</v>
-      </c>
       <c r="O38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Tebby2022.sbml</t>
+          <t>ElMasri2008.sbml</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Tebby2022_Pb_Human</t>
+          <t>ElMasri2008_As_Human</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Tebby 2022</t>
+          <t>ElMasri 2008</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2778,53 +2778,53 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Tebby2022/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/ElMasri2008/summary.md</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Lumen;Gut;Liver;Lung;Arterial;Venous;Rest;Urine</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L39" t="n">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="M39" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="N39" t="n">
-        <v>5</v>
+        <v>107</v>
       </c>
       <c r="O39" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Clewell1999.sbml</t>
+          <t>Carrier2001.sbml</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Clewell_Hg_Human</t>
+          <t>Carrier2001_Hg_Human</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Clewell 1999</t>
+          <t>Carrier 2001</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2839,53 +2839,53 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Carrier2001/summary.md</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
+          <t>GI;Blood;Rest;Hair;Liver</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K40" t="n">
         <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="M40" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="N40" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="O40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Tonnelier.sbml</t>
+          <t>Clewell1999.sbml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Tonnelier2012_Chlorpyrifos_Human</t>
+          <t>Clewell_Hg_Human</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Tonnelier</t>
+          <t>Clewell 1999</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2895,58 +2895,58 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Tonnelier/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Clewell1999/summary.md</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>AbsorptionCompartment;PV;Liver;SystCompartment;RenalExcretion</t>
+          <t>Gut_lumen;Gut;Liver;Red_Blood_Cell;Plasma;Rest;Feces</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I41" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K41" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="M41" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="N41" t="n">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="O41" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Pouillot2022.sbml</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Chen_Fenitrothion_Human</t>
+          <t>Pouillot2022_Cd_Human</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Pouillot 2022</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2956,58 +2956,58 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Chen/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/Pouillot2022/summary.md</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;Rest</t>
+          <t>GI;Intestinal_Tissue;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake;Feces;Urine</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I42" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K42" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="M42" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="N42" t="n">
-        <v>88</v>
+        <v>8</v>
       </c>
       <c r="O42" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Wei.sbml</t>
+          <t>KjellstromNordberg1978.sbml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Wei_Permethrin_Human</t>
+          <t>KjellstromNordberg1978_Cd_Human</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Wei</t>
+          <t>KjellstromNordberg 1978</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3017,58 +3017,58 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Heavy Metals</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Wei/summary.md</t>
+          <t>./models/oral/Heavy%20Metals/KjellstromNordberg1978/summary.md</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;Liver;Blood;RestVC;RestT;Fecal;Urine;ExcretionCompartment</t>
+          <t>GI;Intestinal_Tissue;Plasma;Red_Blood_Cell;Metallothionein;Rest;Daily_Uptake;Feces;Urine</t>
         </is>
       </c>
       <c r="H43" t="n">
         <v>9</v>
       </c>
       <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
         <v>9</v>
       </c>
-      <c r="J43" t="n">
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>12</v>
+      </c>
+      <c r="M43" t="n">
         <v>11</v>
       </c>
-      <c r="K43" t="n">
-        <v>11</v>
-      </c>
-      <c r="L43" t="n">
-        <v>31</v>
-      </c>
-      <c r="M43" t="n">
-        <v>31</v>
-      </c>
       <c r="N43" t="n">
-        <v>104</v>
+        <v>14</v>
       </c>
       <c r="O43" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Bouchard.sbml</t>
+          <t>Mukherjee.sbml</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Bouchard2010_Chlorpyrifos_Human</t>
+          <t>Mukherjee2014_Human_PBK</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bouchard</t>
+          <t>Mukherjee</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3078,58 +3078,58 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Bouchard/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mukherjee/summary.md</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Gut;Blood;Rest</t>
+          <t>GILumen;Fast;Slow;Colon;Gut;Liver;Blood;Rest;Bile;Feces;Stomach;Spleen</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="K44" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="M44" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O44" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Moerenhout.sbml</t>
+          <t>Notenboom.sbml</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Moerenhout2022_Pesticides_Human</t>
+          <t>Notenboom2023_DON_Human</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Moerenhout</t>
+          <t>Notenboom</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3139,58 +3139,58 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moerenhout/summary.md</t>
+          <t>./models/oral/Mycotoxins/Notenboom/summary.md</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Blood;Liver;Kidney;Rest;Urine;Feces</t>
+          <t>Lumen;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="M45" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="O45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Moreau_Deltamethrin.sbml</t>
+          <t>Mendez_Catala.sbml</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>Mandez_Catal_2021_Human_PBK</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl</t>
+          <t>Mendez_Catala</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3200,58 +3200,58 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/Mycotoxins/Mendez_Catala/summary.md</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;LI1;SITissue;Liver;Blood;Rest;Feaces</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I46" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K46" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="M46" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="O46" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl.sbml</t>
+          <t>Gilbert_Sandoval.sbml</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl_Human</t>
+          <t>GilbertSandoval</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Moreau_Carbaryl</t>
+          <t>Gilbert_Sandoval</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3261,58 +3261,58 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Moreau/summary.md</t>
+          <t>./models/oral/Mycotoxins/Gilbert_Sandoval/summary.md</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
+          <t>Stomach;SI1;SI2;SI3;SI4;SI5;SI6;SI7;Colon;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I47" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="K47" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="M47" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="O47" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mallick.sbml</t>
+          <t>Wang.sbml</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Mallick2020_Pyrethroids_Human</t>
+          <t>Wang2023_DON_Human</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mallick</t>
+          <t>Wang</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3322,58 +3322,58 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Mycotoxins</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Mallick/summary.md</t>
+          <t>./models/oral/Mycotoxins/Wang/summary.md</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Lumen;Gut;Liver;Plasma;RestPlasma;RestTissue</t>
+          <t>Stomach;Jejunum;Ileum;LargeLumen;Liver;Blood;Rest;IntestinalTissue</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I48" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K48" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L48" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="M48" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="N48" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O48" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Zhao.sbml</t>
+          <t>Loizou.sbml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Zhao2019_Chlorpyrifos_Human</t>
+          <t>Loizou2022_BPA_Human</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Zhao</t>
+          <t>Loizou</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3383,58 +3383,58 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zhao/summary.md</t>
+          <t>./models/oral/Bisphenols/Loizou/summary.md</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Gut;Liver;Blood;Rest</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I49" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K49" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="M49" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="O49" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Zwartsen.sbml</t>
+          <t>Teeguarden.sbml</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Zwartsen_2025_Chlorpyrifos_Human</t>
+          <t>Teeguarden2005_BPA_Human</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Zwartsen</t>
+          <t>Teeguarden</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3444,58 +3444,58 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Zwartsen/summary.md</t>
+          <t>./models/oral/Bisphenols/Teeguarden/summary.md</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>StomachLumen;IntestineLumen;Liver;Blood;Rest</t>
+          <t>GILumen;Liver;Blood;Rest;Feces</t>
         </is>
       </c>
       <c r="H50" t="n">
         <v>5</v>
       </c>
       <c r="I50" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
         <v>7</v>
       </c>
       <c r="K50" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L50" t="n">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="M50" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="O50" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Godin.sbml</t>
+          <t>Shin.sbml</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Godin_Pyrethroid_Human</t>
+          <t>Shin2004_BPA_Human</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Godin</t>
+          <t>Shin</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3505,58 +3505,58 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Godin/summary.md</t>
+          <t>./models/oral/Bisphenols/Shin/summary.md</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Stomach;Intestinal;LiverVC;LiverIC;Blood;RestVC;RestIC;Fecal</t>
+          <t>Stomach;IntestinalLumen;Spleen;SmallIntestine;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H51" t="n">
+        <v>7</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
         <v>8</v>
       </c>
-      <c r="I51" t="n">
-        <v>8</v>
-      </c>
-      <c r="J51" t="n">
-        <v>10</v>
-      </c>
       <c r="K51" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L51" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="M51" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="O51" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Timchalk.sbml</t>
+          <t>Christensen.sbml</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Timchalk2002_Chlorpyrifos_Human</t>
+          <t>Christensen2013_BPA_Human</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Timchalk</t>
+          <t>Christensen</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3566,58 +3566,58 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Pesticides</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>./models/oral/Pesticides/Timchalk/summary.md</t>
+          <t>./models/oral/Bisphenols/Christensen/summary.md</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Liver;Blood;Rest</t>
+          <t>Stomach;Blood;Bladder</t>
         </is>
       </c>
       <c r="H52" t="n">
         <v>3</v>
       </c>
       <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
         <v>3</v>
       </c>
-      <c r="J52" t="n">
-        <v>5</v>
-      </c>
       <c r="K52" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L52" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="M52" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="O52" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Chen.sbml</t>
+          <t>Sharma.sbml</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Chen2022_PFOS_Human</t>
+          <t>Sharma2018_BPA_Human</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Sharma</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3627,58 +3627,58 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Chen/summary.md</t>
+          <t>./models/oral/Bisphenols/Sharma/summary.md</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H53" t="n">
+        <v>5</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
+        <v>8</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="n">
+        <v>37</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" t="n">
         <v>6</v>
-      </c>
-      <c r="I53" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" t="n">
-        <v>6</v>
-      </c>
-      <c r="K53" t="n">
-        <v>0</v>
-      </c>
-      <c r="L53" t="n">
-        <v>29</v>
-      </c>
-      <c r="M53" t="n">
-        <v>0</v>
-      </c>
-      <c r="N53" t="n">
-        <v>0</v>
-      </c>
-      <c r="O53" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ChouLin.sbml</t>
+          <t>Karrer.sbml</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Chou_Lin2021_PFOS_Human</t>
+          <t>Karrer2018_BPA_Human</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ChouLin</t>
+          <t>Karrer</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3688,58 +3688,58 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/ChouLin/summary.md</t>
+          <t>./models/oral/Bisphenols/Karrer/summary.md</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
       </c>
       <c r="L54" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="M54" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N54" t="n">
         <v>0</v>
       </c>
       <c r="O54" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Husoy.sbml</t>
+          <t>Yang.sbml</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Husoy2024_PFOA_Human</t>
+          <t>Yang2015_BPA_Human</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Husoy</t>
+          <t>Yang</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3749,58 +3749,58 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Husoy/summary.md</t>
+          <t>./models/oral/Bisphenols/Yang/summary.md</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest;Feces</t>
+          <t>Stomach;SI;Liver;Plasma;Rest;GILumen;Feces</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I55" t="n">
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L55" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="M55" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N55" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O55" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Worley.sbml</t>
+          <t>Mielke.sbml</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Worley2017_PFOA_Human</t>
+          <t>Mielke2009_BPA_Human</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Worley</t>
+          <t>Mielke</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3810,21 +3810,21 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Worley/summary.md</t>
+          <t>./models/oral/Bisphenols/Mielke/summary.md</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Stomach;SI;Liver;Plasma;Rest;Feces</t>
+          <t>Gut;Liver;Blood;Rest</t>
         </is>
       </c>
       <c r="H56" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I56" t="n">
         <v>0</v>
@@ -3836,7 +3836,7 @@
         <v>0</v>
       </c>
       <c r="L56" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="M56" t="n">
         <v>0</v>
@@ -3845,7 +3845,7 @@
         <v>0</v>
       </c>
       <c r="O56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Deepika2021_PFOS_Human</t>
+          <t>Deepika2022_BPA_Human</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3871,33 +3871,33 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Deepika/summary.md</t>
+          <t>./models/oral/Bisphenols/Deepika/summary.md</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Stomach;Liver;Plasma;Gut;Rest</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
       </c>
       <c r="L57" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="M57" t="n">
         <v>0</v>
@@ -3906,23 +3906,23 @@
         <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Loccisano.sbml</t>
+          <t>Moreau.sbml</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Loccisano2011_PFAS_Human</t>
+          <t>Moreau2025_BPA_Human</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Loccisano</t>
+          <t>Moreau</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3932,42 +3932,42 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>PFAS</t>
+          <t>Bisphenols</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>./models/oral/PFAS/Loccisano/summary.md</t>
+          <t>./models/oral/Bisphenols/Moreau/summary.md</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>GI;Liver;Plasma;Rest</t>
+          <t>Stomach;GITissue;Duodenum;Liver;Plasma;Rest;Urine</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
       </c>
       <c r="L58" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="M58" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O58" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 395cadf with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -1280,7 +1280,7 @@
         <v>3</v>
       </c>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
         <v>1</v>
@@ -1341,7 +1341,7 @@
         <v>3</v>
       </c>
       <c r="N15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
         <v>1</v>
@@ -1402,10 +1402,10 @@
         <v>3</v>
       </c>
       <c r="N16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Deployed 024f274 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/models/models_overview.xlsx
+++ b/models/models_overview.xlsx
@@ -1274,10 +1274,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>

</xml_diff>